<commit_message>
ÚLTIMA SESSÃO TORMENTA RICHARD
</commit_message>
<xml_diff>
--- a/Fichas/Tormenta/Ficha Cleber.xlsx
+++ b/Fichas/Tormenta/Ficha Cleber.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7755"/>
+    <workbookView windowWidth="20490" windowHeight="7635" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Clebina" sheetId="1" r:id="rId1"/>
@@ -969,7 +969,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="189">
   <si>
     <t>Atributos</t>
   </si>
@@ -1263,6 +1263,9 @@
   </si>
   <si>
     <t>Controlar Madeira</t>
+  </si>
+  <si>
+    <t>disc</t>
   </si>
   <si>
     <t>Enxame de Pesteste</t>
@@ -1618,10 +1621,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="178" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="179" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="28">
     <font>
@@ -1673,83 +1676,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -1766,12 +1692,21 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF3F3F76"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Aptos Narrow"/>
@@ -1786,8 +1721,76 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="13"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="3"/>
       <name val="Aptos Narrow"/>
       <charset val="134"/>
@@ -1803,10 +1806,10 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="Aptos Narrow"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1828,7 +1831,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1849,7 +1852,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1861,13 +1906,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1879,7 +1930,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1891,7 +1948,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1903,55 +2014,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1963,73 +2038,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2552,35 +2561,17 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
       </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
       </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
       </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2600,6 +2591,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -2607,30 +2613,6 @@
       </top>
       <bottom style="double">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2649,155 +2631,182 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="45" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="40" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="43" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="42" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="42" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="45" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="39" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="39" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="43" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="38" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="43" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="44" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="44" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="41" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="41" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="39" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="38" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3003,6 +3012,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3079,54 +3089,54 @@
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="60% - Accent6" xfId="1" builtinId="52"/>
-    <cellStyle name="40% - Accent6" xfId="2" builtinId="51"/>
-    <cellStyle name="60% - Accent5" xfId="3" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="4" builtinId="49"/>
-    <cellStyle name="40% - Accent5" xfId="5" builtinId="47"/>
-    <cellStyle name="20% - Accent5" xfId="6" builtinId="46"/>
-    <cellStyle name="60% - Accent4" xfId="7" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="8" builtinId="45"/>
-    <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
-    <cellStyle name="Accent4" xfId="10" builtinId="41"/>
-    <cellStyle name="Linked Cell" xfId="11" builtinId="24"/>
-    <cellStyle name="40% - Accent3" xfId="12" builtinId="39"/>
-    <cellStyle name="60% - Accent2" xfId="13" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="14" builtinId="37"/>
-    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
-    <cellStyle name="20% - Accent2" xfId="16" builtinId="34"/>
-    <cellStyle name="Accent2" xfId="17" builtinId="33"/>
-    <cellStyle name="40% - Accent1" xfId="18" builtinId="31"/>
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30"/>
-    <cellStyle name="Accent1" xfId="20" builtinId="29"/>
-    <cellStyle name="Neutral" xfId="21" builtinId="28"/>
-    <cellStyle name="60% - Accent1" xfId="22" builtinId="32"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="20% - Accent4" xfId="24" builtinId="42"/>
-    <cellStyle name="Total" xfId="25" builtinId="25"/>
-    <cellStyle name="Output" xfId="26" builtinId="21"/>
-    <cellStyle name="Currency" xfId="27" builtinId="4"/>
-    <cellStyle name="20% - Accent3" xfId="28" builtinId="38"/>
-    <cellStyle name="Note" xfId="29" builtinId="10"/>
-    <cellStyle name="Input" xfId="30" builtinId="20"/>
-    <cellStyle name="Heading 4" xfId="31" builtinId="19"/>
-    <cellStyle name="Calculation" xfId="32" builtinId="22"/>
-    <cellStyle name="Good" xfId="33" builtinId="26"/>
-    <cellStyle name="Heading 3" xfId="34" builtinId="18"/>
-    <cellStyle name="CExplanatory Text" xfId="35" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="36" builtinId="16"/>
-    <cellStyle name="Comma [0]" xfId="37" builtinId="6"/>
-    <cellStyle name="20% - Accent6" xfId="38" builtinId="50"/>
-    <cellStyle name="Title" xfId="39" builtinId="15"/>
-    <cellStyle name="Currency [0]" xfId="40" builtinId="7"/>
-    <cellStyle name="Warning Text" xfId="41" builtinId="11"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9"/>
-    <cellStyle name="Heading 2" xfId="43" builtinId="17"/>
-    <cellStyle name="Comma" xfId="44" builtinId="3"/>
-    <cellStyle name="Check Cell" xfId="45" builtinId="23"/>
-    <cellStyle name="60% - Accent3" xfId="46" builtinId="40"/>
-    <cellStyle name="Percent" xfId="47" builtinId="5"/>
-    <cellStyle name="Hyperlink" xfId="48" builtinId="8"/>
+    <cellStyle name="60% - Ênfase 6" xfId="1" builtinId="52"/>
+    <cellStyle name="40% - Ênfase 6" xfId="2" builtinId="51"/>
+    <cellStyle name="20% - Ênfase 6" xfId="3" builtinId="50"/>
+    <cellStyle name="40% - Ênfase 5" xfId="4" builtinId="47"/>
+    <cellStyle name="Ênfase 5" xfId="5" builtinId="45"/>
+    <cellStyle name="Ênfase 4" xfId="6" builtinId="41"/>
+    <cellStyle name="Título 4" xfId="7" builtinId="19"/>
+    <cellStyle name="60% - Ênfase 3" xfId="8" builtinId="40"/>
+    <cellStyle name="20% - Ênfase 3" xfId="9" builtinId="38"/>
+    <cellStyle name="Ênfase 3" xfId="10" builtinId="37"/>
+    <cellStyle name="Título 3" xfId="11" builtinId="18"/>
+    <cellStyle name="60% - Ênfase 2" xfId="12" builtinId="36"/>
+    <cellStyle name="Célula de Verificação" xfId="13" builtinId="23"/>
+    <cellStyle name="40% - Ênfase 2" xfId="14" builtinId="35"/>
+    <cellStyle name="60% - Ênfase 5" xfId="15" builtinId="48"/>
+    <cellStyle name="Ênfase 2" xfId="16" builtinId="33"/>
+    <cellStyle name="Ênfase 6" xfId="17" builtinId="49"/>
+    <cellStyle name="40% - Ênfase 1" xfId="18" builtinId="31"/>
+    <cellStyle name="20% - Ênfase 1" xfId="19" builtinId="30"/>
+    <cellStyle name="60% - Ênfase 4" xfId="20" builtinId="44"/>
+    <cellStyle name="Ênfase 1" xfId="21" builtinId="29"/>
+    <cellStyle name="40% - Ênfase 4" xfId="22" builtinId="43"/>
+    <cellStyle name="Ruim" xfId="23" builtinId="27"/>
+    <cellStyle name="20% - Ênfase 4" xfId="24" builtinId="42"/>
+    <cellStyle name="Saída" xfId="25" builtinId="21"/>
+    <cellStyle name="Hyperlink seguido" xfId="26" builtinId="9"/>
+    <cellStyle name="Moeda [0]" xfId="27" builtinId="7"/>
+    <cellStyle name="Total" xfId="28" builtinId="25"/>
+    <cellStyle name="Bom" xfId="29" builtinId="26"/>
+    <cellStyle name="40% - Ênfase 3" xfId="30" builtinId="39"/>
+    <cellStyle name="Texto de Aviso" xfId="31" builtinId="11"/>
+    <cellStyle name="Cálculo" xfId="32" builtinId="22"/>
+    <cellStyle name="Entrada" xfId="33" builtinId="20"/>
+    <cellStyle name="Texto Explicativo" xfId="34" builtinId="53"/>
+    <cellStyle name="Título 1" xfId="35" builtinId="16"/>
+    <cellStyle name="Título" xfId="36" builtinId="15"/>
+    <cellStyle name="Observação" xfId="37" builtinId="10"/>
+    <cellStyle name="20% - Ênfase 2" xfId="38" builtinId="34"/>
+    <cellStyle name="60% - Ênfase 1" xfId="39" builtinId="32"/>
+    <cellStyle name="Título 2" xfId="40" builtinId="17"/>
+    <cellStyle name="Hyperlink" xfId="41" builtinId="8"/>
+    <cellStyle name="Célula Vinculada" xfId="42" builtinId="24"/>
+    <cellStyle name="Comma" xfId="43" builtinId="3"/>
+    <cellStyle name="Porcentagem" xfId="44" builtinId="5"/>
+    <cellStyle name="Neutro" xfId="45" builtinId="28"/>
+    <cellStyle name="20% - Ênfase 5" xfId="46" builtinId="46"/>
+    <cellStyle name="Moeda" xfId="47" builtinId="4"/>
+    <cellStyle name="Comma [0]" xfId="48" builtinId="6"/>
   </cellStyles>
   <dxfs count="28">
     <dxf>
@@ -4396,19 +4406,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="B1:N41"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="12.4266666666667" customWidth="1"/>
-    <col min="3" max="3" width="6.14222222222222" customWidth="1"/>
-    <col min="4" max="4" width="13.2844444444444" customWidth="1"/>
-    <col min="6" max="6" width="14.5688888888889" customWidth="1"/>
-    <col min="7" max="8" width="7.85333333333333" customWidth="1"/>
+    <col min="2" max="2" width="12.425" customWidth="1"/>
+    <col min="3" max="3" width="6.14166666666667" customWidth="1"/>
+    <col min="4" max="4" width="13.2833333333333" customWidth="1"/>
+    <col min="6" max="6" width="14.5666666666667" customWidth="1"/>
+    <col min="7" max="8" width="7.85" customWidth="1"/>
     <col min="9" max="9" width="6" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="14" max="14" width="36.4266666666667" customWidth="1"/>
+    <col min="14" max="14" width="36.425" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25"/>
+    <row r="1" ht="15.75"/>
     <row r="2" ht="15.75" customHeight="1" spans="2:14">
       <c r="B2" s="35" t="s">
         <v>0</v>
@@ -4449,7 +4459,7 @@
       </c>
       <c r="G3" s="27">
         <f>H3-L25-SUM(L4:L22)</f>
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H3" s="39">
         <f>'uns dados aí'!M2+((G2-1)*'uns dados aí'!C12)</f>
@@ -4494,7 +4504,9 @@
       <c r="K4" s="41">
         <v>1</v>
       </c>
-      <c r="L4" s="29"/>
+      <c r="L4" s="29">
+        <v>12</v>
+      </c>
       <c r="M4" s="29"/>
       <c r="N4" s="42"/>
     </row>
@@ -4517,11 +4529,13 @@
         <f>10+D4+C16</f>
         <v>22</v>
       </c>
-      <c r="H5" s="89"/>
+      <c r="H5" s="90"/>
       <c r="K5" s="38">
         <v>2</v>
       </c>
-      <c r="L5" s="27"/>
+      <c r="L5" s="27">
+        <v>-6</v>
+      </c>
       <c r="M5" s="27"/>
       <c r="N5" s="39"/>
     </row>
@@ -4544,7 +4558,7 @@
         <f>G5+Perícias!J12</f>
         <v>27</v>
       </c>
-      <c r="H6" s="90"/>
+      <c r="H6" s="91"/>
       <c r="K6" s="41">
         <v>3</v>
       </c>
@@ -4571,7 +4585,7 @@
         <f>Perícias!J27+Perícias!J21</f>
         <v>17</v>
       </c>
-      <c r="H7" s="89"/>
+      <c r="H7" s="90"/>
       <c r="K7" s="38">
         <v>4</v>
       </c>
@@ -4579,7 +4593,7 @@
       <c r="M7" s="27"/>
       <c r="N7" s="39"/>
     </row>
-    <row r="8" ht="17.25" spans="2:14">
+    <row r="8" ht="15.75" spans="2:14">
       <c r="B8" s="45" t="s">
         <v>16</v>
       </c>
@@ -4594,10 +4608,10 @@
       <c r="F8" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="91">
+      <c r="G8" s="92">
         <v>0.5</v>
       </c>
-      <c r="H8" s="92"/>
+      <c r="H8" s="93"/>
       <c r="K8" s="41">
         <v>5</v>
       </c>
@@ -4605,12 +4619,12 @@
       <c r="M8" s="29"/>
       <c r="N8" s="42"/>
     </row>
-    <row r="9" spans="6:14">
+    <row r="9" ht="15.75" spans="6:14">
       <c r="F9" s="38" t="s">
         <v>18</v>
       </c>
       <c r="G9" s="27">
-        <v>220</v>
+        <v>18</v>
       </c>
       <c r="H9" s="39"/>
       <c r="K9" s="38">
@@ -4620,7 +4634,7 @@
       <c r="M9" s="27"/>
       <c r="N9" s="39"/>
     </row>
-    <row r="10" ht="17.25" spans="6:14">
+    <row r="10" ht="15.75" spans="6:14">
       <c r="F10" s="45" t="s">
         <v>19</v>
       </c>
@@ -4635,7 +4649,7 @@
       <c r="M10" s="29"/>
       <c r="N10" s="42"/>
     </row>
-    <row r="11" ht="18" spans="11:14">
+    <row r="11" ht="16.5" spans="11:14">
       <c r="K11" s="38">
         <v>8</v>
       </c>
@@ -4643,17 +4657,17 @@
       <c r="M11" s="27"/>
       <c r="N11" s="39"/>
     </row>
-    <row r="12" ht="18" spans="2:14">
-      <c r="B12" s="71" t="s">
+    <row r="12" ht="16.5" spans="2:14">
+      <c r="B12" s="72" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="72"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="72"/>
-      <c r="F12" s="72"/>
-      <c r="G12" s="72"/>
-      <c r="H12" s="72"/>
-      <c r="I12" s="73"/>
+      <c r="C12" s="73"/>
+      <c r="D12" s="73"/>
+      <c r="E12" s="73"/>
+      <c r="F12" s="73"/>
+      <c r="G12" s="73"/>
+      <c r="H12" s="73"/>
+      <c r="I12" s="74"/>
       <c r="K12" s="41">
         <v>9</v>
       </c>
@@ -4661,8 +4675,8 @@
       <c r="M12" s="29"/>
       <c r="N12" s="42"/>
     </row>
-    <row r="13" ht="18" spans="2:14">
-      <c r="B13" s="88"/>
+    <row r="13" ht="16.5" spans="2:14">
+      <c r="B13" s="89"/>
       <c r="K13" s="38">
         <v>10</v>
       </c>
@@ -4670,7 +4684,7 @@
       <c r="M13" s="27"/>
       <c r="N13" s="39"/>
     </row>
-    <row r="14" ht="17.25" spans="2:14">
+    <row r="14" ht="15.75" spans="2:14">
       <c r="B14" s="35" t="s">
         <v>21</v>
       </c>
@@ -4718,7 +4732,7 @@
       <c r="M15" s="27"/>
       <c r="N15" s="39"/>
     </row>
-    <row r="16" ht="17.25" spans="2:14">
+    <row r="16" ht="30.75" spans="2:14">
       <c r="B16" s="45" t="s">
         <v>29</v>
       </c>
@@ -4752,7 +4766,7 @@
       <c r="M16" s="29"/>
       <c r="N16" s="42"/>
     </row>
-    <row r="17" ht="17.25" spans="11:14">
+    <row r="17" ht="15.75" spans="11:14">
       <c r="K17" s="38">
         <v>14</v>
       </c>
@@ -4800,8 +4814,8 @@
       <c r="M22" s="53"/>
       <c r="N22" s="46"/>
     </row>
-    <row r="23" ht="18"/>
-    <row r="24" ht="17.25" spans="11:12">
+    <row r="23" ht="16.5"/>
+    <row r="24" ht="15.75" spans="11:12">
       <c r="K24" s="35" t="s">
         <v>31</v>
       </c>
@@ -4813,13 +4827,13 @@
       </c>
       <c r="L25" s="39"/>
     </row>
-    <row r="26" ht="17.25" spans="11:12">
+    <row r="26" ht="15.75" spans="11:12">
       <c r="K26" s="45" t="s">
         <v>7</v>
       </c>
       <c r="L26" s="46"/>
     </row>
-    <row r="27" ht="17.25"/>
+    <row r="27" ht="15.75"/>
     <row r="41" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="13">
@@ -4854,35 +4868,35 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:O23"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="12" max="12" width="19.7111111111111" customWidth="1"/>
-    <col min="13" max="13" width="12.2844444444444" customWidth="1"/>
-    <col min="14" max="14" width="12.1422222222222" customWidth="1"/>
+    <col min="12" max="12" width="19.7083333333333" customWidth="1"/>
+    <col min="13" max="13" width="12.2833333333333" customWidth="1"/>
+    <col min="14" max="14" width="12.1416666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" spans="1:15">
-      <c r="A1" s="71" t="s">
+    <row r="1" ht="16.5" spans="1:15">
+      <c r="A1" s="72" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="73"/>
-      <c r="I1" s="71" t="s">
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="74"/>
+      <c r="I1" s="72" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="73"/>
-    </row>
-    <row r="2" ht="18"/>
-    <row r="3" ht="17.25" spans="2:13">
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="74"/>
+    </row>
+    <row r="2" ht="16.5"/>
+    <row r="3" ht="15.75" spans="2:13">
       <c r="B3" s="35" t="s">
         <v>34</v>
       </c>
@@ -4892,17 +4906,17 @@
       </c>
       <c r="E3" s="48"/>
       <c r="F3" s="36"/>
-      <c r="K3" s="75" t="s">
+      <c r="K3" s="76" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="76" t="s">
+      <c r="L3" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="M3" s="84" t="s">
+      <c r="M3" s="85" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="2:13">
+    <row r="4" customHeight="1" spans="2:13">
       <c r="B4" s="38" t="s">
         <v>38</v>
       </c>
@@ -4914,15 +4928,15 @@
       <c r="F4" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="77" t="s">
+      <c r="K4" s="78" t="s">
         <v>41</v>
       </c>
-      <c r="L4" s="78" t="s">
+      <c r="L4" s="79" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="85"/>
-    </row>
-    <row r="5" ht="15" customHeight="1" spans="2:13">
+      <c r="M4" s="86"/>
+    </row>
+    <row r="5" customHeight="1" spans="2:13">
       <c r="B5" s="41" t="s">
         <v>43</v>
       </c>
@@ -4934,15 +4948,15 @@
       <c r="F5" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="K5" s="79" t="s">
+      <c r="K5" s="80" t="s">
         <v>41</v>
       </c>
-      <c r="L5" s="80" t="s">
+      <c r="L5" s="81" t="s">
         <v>45</v>
       </c>
-      <c r="M5" s="86"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" spans="2:13">
+      <c r="M5" s="87"/>
+    </row>
+    <row r="6" customHeight="1" spans="2:13">
       <c r="B6" s="38" t="s">
         <v>46</v>
       </c>
@@ -4954,13 +4968,13 @@
       <c r="F6" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K6" s="77" t="s">
+      <c r="K6" s="78" t="s">
         <v>41</v>
       </c>
-      <c r="L6" s="78" t="s">
+      <c r="L6" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="M6" s="85"/>
+      <c r="M6" s="86"/>
     </row>
     <row r="7" spans="2:13">
       <c r="B7" s="41" t="s">
@@ -4974,13 +4988,13 @@
       <c r="F7" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="K7" s="79" t="s">
+      <c r="K7" s="80" t="s">
         <v>51</v>
       </c>
-      <c r="L7" s="80" t="s">
+      <c r="L7" s="81" t="s">
         <v>52</v>
       </c>
-      <c r="M7" s="86"/>
+      <c r="M7" s="87"/>
     </row>
     <row r="8" spans="2:13">
       <c r="B8" s="38" t="s">
@@ -4994,13 +5008,13 @@
       <c r="F8" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K8" s="77" t="s">
+      <c r="K8" s="78" t="s">
         <v>55</v>
       </c>
-      <c r="L8" s="81" t="s">
+      <c r="L8" s="82" t="s">
         <v>56</v>
       </c>
-      <c r="M8" s="85"/>
+      <c r="M8" s="86"/>
     </row>
     <row r="9" spans="2:13">
       <c r="B9" s="41" t="s">
@@ -5014,11 +5028,11 @@
       <c r="F9" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="79"/>
-      <c r="L9" s="80"/>
-      <c r="M9" s="86"/>
-    </row>
-    <row r="10" ht="15" customHeight="1" spans="2:13">
+      <c r="K9" s="80"/>
+      <c r="L9" s="81"/>
+      <c r="M9" s="87"/>
+    </row>
+    <row r="10" customHeight="1" spans="2:13">
       <c r="B10" s="38" t="s">
         <v>59</v>
       </c>
@@ -5030,9 +5044,9 @@
       <c r="F10" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K10" s="77"/>
-      <c r="L10" s="78"/>
-      <c r="M10" s="85"/>
+      <c r="K10" s="78"/>
+      <c r="L10" s="79"/>
+      <c r="M10" s="86"/>
     </row>
     <row r="11" spans="2:13">
       <c r="B11" s="41" t="s">
@@ -5046,9 +5060,9 @@
       <c r="F11" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="79"/>
-      <c r="L11" s="80"/>
-      <c r="M11" s="86"/>
+      <c r="K11" s="80"/>
+      <c r="L11" s="81"/>
+      <c r="M11" s="87"/>
     </row>
     <row r="12" spans="2:13">
       <c r="B12" s="38" t="s">
@@ -5062,9 +5076,9 @@
       <c r="F12" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K12" s="77"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="85"/>
+      <c r="K12" s="78"/>
+      <c r="L12" s="79"/>
+      <c r="M12" s="86"/>
     </row>
     <row r="13" spans="2:13">
       <c r="B13" s="41" t="s">
@@ -5078,10 +5092,10 @@
       <c r="F13" s="42" t="s">
         <v>67</v>
       </c>
-      <c r="G13" s="74"/>
-      <c r="K13" s="79"/>
-      <c r="L13" s="80"/>
-      <c r="M13" s="86"/>
+      <c r="G13" s="75"/>
+      <c r="K13" s="80"/>
+      <c r="L13" s="81"/>
+      <c r="M13" s="87"/>
     </row>
     <row r="14" spans="2:13">
       <c r="B14" s="38" t="s">
@@ -5091,9 +5105,9 @@
       <c r="D14" s="27"/>
       <c r="E14" s="27"/>
       <c r="F14" s="39"/>
-      <c r="K14" s="77"/>
-      <c r="L14" s="78"/>
-      <c r="M14" s="85"/>
+      <c r="K14" s="78"/>
+      <c r="L14" s="79"/>
+      <c r="M14" s="86"/>
     </row>
     <row r="15" spans="2:13">
       <c r="B15" s="41" t="s">
@@ -5103,9 +5117,9 @@
       <c r="D15" s="29"/>
       <c r="E15" s="29"/>
       <c r="F15" s="42"/>
-      <c r="K15" s="79"/>
-      <c r="L15" s="80"/>
-      <c r="M15" s="86"/>
+      <c r="K15" s="80"/>
+      <c r="L15" s="81"/>
+      <c r="M15" s="87"/>
     </row>
     <row r="16" spans="2:13">
       <c r="B16" s="38" t="s">
@@ -5115,9 +5129,9 @@
       <c r="D16" s="27"/>
       <c r="E16" s="27"/>
       <c r="F16" s="39"/>
-      <c r="K16" s="77"/>
-      <c r="L16" s="78"/>
-      <c r="M16" s="85"/>
+      <c r="K16" s="78"/>
+      <c r="L16" s="79"/>
+      <c r="M16" s="86"/>
     </row>
     <row r="17" spans="2:13">
       <c r="B17" s="41" t="s">
@@ -5127,9 +5141,9 @@
       <c r="D17" s="29"/>
       <c r="E17" s="29"/>
       <c r="F17" s="42"/>
-      <c r="K17" s="79"/>
-      <c r="L17" s="80"/>
-      <c r="M17" s="86"/>
+      <c r="K17" s="80"/>
+      <c r="L17" s="81"/>
+      <c r="M17" s="87"/>
     </row>
     <row r="18" spans="2:13">
       <c r="B18" s="38" t="s">
@@ -5139,9 +5153,9 @@
       <c r="D18" s="27"/>
       <c r="E18" s="27"/>
       <c r="F18" s="39"/>
-      <c r="K18" s="77"/>
-      <c r="L18" s="78"/>
-      <c r="M18" s="85"/>
+      <c r="K18" s="78"/>
+      <c r="L18" s="79"/>
+      <c r="M18" s="86"/>
     </row>
     <row r="19" spans="2:13">
       <c r="B19" s="41" t="s">
@@ -5151,9 +5165,9 @@
       <c r="D19" s="29"/>
       <c r="E19" s="29"/>
       <c r="F19" s="42"/>
-      <c r="K19" s="79"/>
-      <c r="L19" s="80"/>
-      <c r="M19" s="86"/>
+      <c r="K19" s="80"/>
+      <c r="L19" s="81"/>
+      <c r="M19" s="87"/>
     </row>
     <row r="20" spans="2:13">
       <c r="B20" s="38" t="s">
@@ -5163,9 +5177,9 @@
       <c r="D20" s="27"/>
       <c r="E20" s="27"/>
       <c r="F20" s="39"/>
-      <c r="K20" s="77"/>
-      <c r="L20" s="78"/>
-      <c r="M20" s="85"/>
+      <c r="K20" s="78"/>
+      <c r="L20" s="79"/>
+      <c r="M20" s="86"/>
     </row>
     <row r="21" spans="2:13">
       <c r="B21" s="41" t="s">
@@ -5175,11 +5189,11 @@
       <c r="D21" s="29"/>
       <c r="E21" s="29"/>
       <c r="F21" s="42"/>
-      <c r="K21" s="79"/>
-      <c r="L21" s="80"/>
-      <c r="M21" s="86"/>
-    </row>
-    <row r="22" ht="17.25" spans="2:13">
+      <c r="K21" s="80"/>
+      <c r="L21" s="81"/>
+      <c r="M21" s="87"/>
+    </row>
+    <row r="22" ht="15.75" spans="2:13">
       <c r="B22" s="43" t="s">
         <v>76</v>
       </c>
@@ -5187,11 +5201,11 @@
       <c r="D22" s="50"/>
       <c r="E22" s="50"/>
       <c r="F22" s="44"/>
-      <c r="K22" s="82"/>
-      <c r="L22" s="83"/>
-      <c r="M22" s="87"/>
-    </row>
-    <row r="23" ht="17.25"/>
+      <c r="K22" s="83"/>
+      <c r="L22" s="84"/>
+      <c r="M22" s="88"/>
+    </row>
+    <row r="23" ht="15.75"/>
   </sheetData>
   <mergeCells count="42">
     <mergeCell ref="A1:G1"/>
@@ -5247,14 +5261,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="B1:H32"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="7"/>
   <cols>
-    <col min="2" max="2" width="13.8533333333333" customWidth="1"/>
-    <col min="7" max="7" width="8.42666666666667" customWidth="1"/>
+    <col min="2" max="2" width="13.85" customWidth="1"/>
+    <col min="7" max="7" width="8.425" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25"/>
-    <row r="2" ht="17.25" spans="2:8">
+    <row r="1" ht="15.75"/>
+    <row r="2" ht="15.75" spans="2:8">
       <c r="B2" s="35" t="s">
         <v>0</v>
       </c>
@@ -5272,7 +5286,7 @@
       </c>
       <c r="H2" s="65"/>
     </row>
-    <row r="3" ht="17.25" spans="2:8">
+    <row r="3" ht="15.75" spans="2:8">
       <c r="B3" s="38" t="str">
         <f>Tabela1[[#This Row],[Perícia]]</f>
         <v>Acrobacia</v>
@@ -5283,21 +5297,21 @@
       </c>
       <c r="D3" s="27">
         <f ca="1">RANDBETWEEN(1,20)</f>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E3" s="39">
         <f ca="1">SUM(C3:D3)</f>
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="G3" s="43" t="s">
         <v>80</v>
       </c>
       <c r="H3" s="44">
         <f ca="1">VLOOKUP(G3,B2:E31,4,FALSE)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" ht="17.25" spans="2:5">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" spans="2:5">
       <c r="B4" s="41" t="str">
         <f>Tabela1[[#This Row],[Perícia]]</f>
         <v>Adestramento</v>
@@ -5308,11 +5322,11 @@
       </c>
       <c r="D4" s="29">
         <f ca="1" t="shared" ref="D4:D31" si="0">RANDBETWEEN(1,20)</f>
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E4" s="42">
         <f ca="1" t="shared" ref="E4:E31" si="1">SUM(C4:D4)</f>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="2:5">
@@ -5326,11 +5340,11 @@
       </c>
       <c r="D5" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="E5" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:5">
@@ -5344,11 +5358,11 @@
       </c>
       <c r="D6" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E6" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="2:5">
@@ -5362,11 +5376,11 @@
       </c>
       <c r="D7" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E7" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="2:5">
@@ -5380,11 +5394,11 @@
       </c>
       <c r="D8" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E8" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="2:5">
@@ -5398,11 +5412,11 @@
       </c>
       <c r="D9" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E9" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="2:5">
@@ -5416,11 +5430,11 @@
       </c>
       <c r="D10" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E10" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="2:5">
@@ -5434,11 +5448,11 @@
       </c>
       <c r="D11" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E11" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="2:5">
@@ -5452,11 +5466,11 @@
       </c>
       <c r="D12" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E12" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="2:5">
@@ -5470,11 +5484,11 @@
       </c>
       <c r="D13" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E13" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="2:5">
@@ -5488,11 +5502,11 @@
       </c>
       <c r="D14" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E14" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="2:5">
@@ -5506,11 +5520,11 @@
       </c>
       <c r="D15" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E15" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="2:5">
@@ -5524,11 +5538,11 @@
       </c>
       <c r="D16" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E16" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="2:5">
@@ -5542,11 +5556,11 @@
       </c>
       <c r="D17" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E17" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="2:5">
@@ -5578,11 +5592,11 @@
       </c>
       <c r="D19" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E19" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="2:5">
@@ -5596,11 +5610,11 @@
       </c>
       <c r="D20" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E20" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="2:5">
@@ -5614,11 +5628,11 @@
       </c>
       <c r="D21" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E21" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>8</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="2:5">
@@ -5632,11 +5646,11 @@
       </c>
       <c r="D22" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E22" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="2:5">
@@ -5657,7 +5671,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="2:5">
+    <row r="24" ht="30" spans="2:5">
       <c r="B24" s="41" t="str">
         <f>Tabela1[[#This Row],[Perícia]]</f>
         <v>Ofício (Alquimista)</v>
@@ -5668,11 +5682,11 @@
       </c>
       <c r="D24" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E24" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="2:5">
@@ -5686,14 +5700,14 @@
       </c>
       <c r="D25" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E25" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" ht="30" spans="2:5">
       <c r="B26" s="41" t="str">
         <f>Tabela1[[#This Row],[Perícia]]</f>
         <v>Ofício (Engenhoqueiro)</v>
@@ -5704,11 +5718,11 @@
       </c>
       <c r="D26" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E26" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27" spans="2:5">
@@ -5722,11 +5736,11 @@
       </c>
       <c r="D27" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E27" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="2:5">
@@ -5758,11 +5772,11 @@
       </c>
       <c r="D29" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E29" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="2:5">
@@ -5776,14 +5790,14 @@
       </c>
       <c r="D30" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E30" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="31" ht="17.25" spans="2:5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" ht="15.75" spans="2:5">
       <c r="B31" s="43" t="str">
         <f>Tabela1[[#This Row],[Perícia]]</f>
         <v>Religião</v>
@@ -5794,14 +5808,14 @@
       </c>
       <c r="D31" s="50">
         <f ca="1" t="shared" si="0"/>
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E31" s="44">
         <f ca="1" t="shared" si="1"/>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="32" ht="17.25"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="G2:H2"/>
@@ -5819,17 +5833,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B1:H35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" outlineLevelCol="7"/>
+  <dimension ref="A1:H35"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="7"/>
   <cols>
-    <col min="2" max="2" width="23.2844444444444" customWidth="1"/>
-    <col min="3" max="3" width="15.4266666666667" customWidth="1"/>
-    <col min="4" max="4" width="11.8533333333333" customWidth="1"/>
-    <col min="5" max="5" width="10.5688888888889" customWidth="1"/>
+    <col min="2" max="2" width="23.2833333333333" customWidth="1"/>
+    <col min="3" max="3" width="15.425" customWidth="1"/>
+    <col min="4" max="4" width="11.85" customWidth="1"/>
+    <col min="5" max="5" width="10.5666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25"/>
-    <row r="2" ht="17.25" spans="2:8">
+    <row r="1" ht="15.75"/>
+    <row r="2" ht="15.75" spans="2:8">
       <c r="B2" s="24" t="s">
         <v>81</v>
       </c>
@@ -5839,7 +5853,7 @@
       <c r="D2" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="70" t="s">
+      <c r="E2" s="71" t="s">
         <v>83</v>
       </c>
       <c r="G2" s="35" t="s">
@@ -5861,9 +5875,6 @@
         <f t="shared" ref="E3:E35" si="0">IFERROR(VLOOKUP(D3,$G$3:$H$7,2,FALSE)^2*10,"")</f>
         <v>10</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
       <c r="G3" s="38">
         <v>1</v>
       </c>
@@ -5885,9 +5896,6 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
       <c r="G4" s="41">
         <v>2</v>
       </c>
@@ -5937,7 +5945,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" ht="17.25" spans="2:8">
+    <row r="7" ht="15.75" spans="1:8">
+      <c r="A7" s="69"/>
       <c r="B7" s="68" t="s">
         <v>91</v>
       </c>
@@ -5951,6 +5960,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
+      <c r="F7" s="69"/>
       <c r="G7" s="43">
         <v>5</v>
       </c>
@@ -5958,7 +5968,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" ht="17.25" spans="2:5">
+    <row r="8" ht="15.75" spans="2:5">
       <c r="B8" s="30" t="s">
         <v>92</v>
       </c>
@@ -6033,7 +6043,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:5">
+    <row r="13" spans="2:7">
       <c r="B13" s="68" t="s">
         <v>97</v>
       </c>
@@ -6047,10 +6057,13 @@
         <f t="shared" si="0"/>
         <v>90</v>
       </c>
+      <c r="G13" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="14" spans="2:5">
       <c r="B14" s="30" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C14" s="28" t="s">
         <v>86</v>
@@ -6065,10 +6078,10 @@
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="68" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D15" s="27">
         <v>2</v>
@@ -6080,7 +6093,7 @@
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="30" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C16" s="28" t="s">
         <v>89</v>
@@ -6256,7 +6269,7 @@
       </c>
     </row>
     <row r="35" spans="2:5">
-      <c r="B35" s="69"/>
+      <c r="B35" s="70"/>
       <c r="C35" s="31"/>
       <c r="D35" s="32"/>
       <c r="E35" s="47" t="str">
@@ -6281,17 +6294,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="B1:I35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="21.1422222222222" customWidth="1"/>
-    <col min="4" max="4" width="17.7111111111111" customWidth="1"/>
+    <col min="2" max="2" width="21.1416666666667" customWidth="1"/>
+    <col min="4" max="4" width="17.7083333333333" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25"/>
-    <row r="2" ht="17.25" spans="2:6">
+    <row r="1" ht="15.75"/>
+    <row r="2" ht="15.75" spans="2:6">
       <c r="B2" s="35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C2" s="48"/>
       <c r="D2" s="48"/>
@@ -6309,15 +6322,15 @@
         <v>25</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F3" s="39" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="2:6">
       <c r="B4" s="49" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C4" s="29">
         <v>10</v>
@@ -6332,17 +6345,17 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" ht="17.25" spans="2:6">
+    <row r="5" ht="15.75" spans="2:6">
       <c r="B5" s="43"/>
       <c r="C5" s="50"/>
       <c r="D5" s="50"/>
       <c r="E5" s="64"/>
       <c r="F5" s="44"/>
     </row>
-    <row r="6" ht="18"/>
-    <row r="7" ht="17.25" spans="2:8">
+    <row r="6" ht="16.5"/>
+    <row r="7" ht="15.75" spans="2:8">
       <c r="B7" s="51" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C7" s="52"/>
       <c r="D7" s="52"/>
@@ -6359,13 +6372,13 @@
         <v>26</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E8" s="27" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G8" s="37" t="s">
         <v>36</v>
@@ -6379,37 +6392,37 @@
         <v>30</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D9" s="29"/>
       <c r="E9" s="29"/>
       <c r="F9" s="40"/>
       <c r="G9" s="40" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H9" s="42" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="2:8">
       <c r="B10" s="38" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D10" s="27" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="37">
         <v>2</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H10" s="39" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" spans="2:8">
@@ -6430,7 +6443,7 @@
       <c r="G12" s="37"/>
       <c r="H12" s="39"/>
     </row>
-    <row r="13" ht="17.25" spans="2:8">
+    <row r="13" ht="15.75" spans="2:8">
       <c r="B13" s="45"/>
       <c r="C13" s="53"/>
       <c r="D13" s="53"/>
@@ -6439,10 +6452,10 @@
       <c r="G13" s="66"/>
       <c r="H13" s="46"/>
     </row>
-    <row r="14" ht="18"/>
-    <row r="15" ht="17.25" spans="2:9">
+    <row r="14" ht="16.5"/>
+    <row r="15" ht="15.75" spans="2:9">
       <c r="B15" s="35" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C15" s="48"/>
       <c r="D15" s="48"/>
@@ -6461,27 +6474,27 @@
       </c>
       <c r="D16" s="55"/>
       <c r="E16" s="55" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F16" s="55" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G16" s="55" t="s">
+        <v>105</v>
+      </c>
+      <c r="H16" s="55" t="s">
+        <v>118</v>
+      </c>
+      <c r="I16" s="67" t="s">
         <v>104</v>
-      </c>
-      <c r="H16" s="55" t="s">
-        <v>117</v>
-      </c>
-      <c r="I16" s="67" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="17" spans="2:9">
       <c r="B17" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="C17" s="93" t="s">
         <v>119</v>
+      </c>
+      <c r="C17" s="94" t="s">
+        <v>120</v>
       </c>
       <c r="D17" s="11"/>
       <c r="E17" s="29">
@@ -6504,10 +6517,10 @@
     </row>
     <row r="18" spans="2:9">
       <c r="B18" s="54" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C18" s="55" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D18" s="55"/>
       <c r="E18" s="55">
@@ -6528,10 +6541,10 @@
     </row>
     <row r="19" spans="2:9">
       <c r="B19" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C19" s="11" t="s">
         <v>122</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>121</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="29">
@@ -6552,7 +6565,7 @@
     </row>
     <row r="20" spans="2:9">
       <c r="B20" s="54" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C20" s="55"/>
       <c r="D20" s="55"/>
@@ -6574,7 +6587,7 @@
     </row>
     <row r="21" spans="2:9">
       <c r="B21" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
@@ -6660,7 +6673,7 @@
       <c r="H28" s="55"/>
       <c r="I28" s="67"/>
     </row>
-    <row r="29" ht="17.25" spans="2:9">
+    <row r="29" ht="15.75" spans="2:9">
       <c r="B29" s="7"/>
       <c r="C29" s="56"/>
       <c r="D29" s="56"/>
@@ -6670,11 +6683,11 @@
       <c r="H29" s="53"/>
       <c r="I29" s="46"/>
     </row>
-    <row r="30" ht="17.25"/>
-    <row r="31" ht="17.25"/>
-    <row r="32" ht="17.25" spans="2:4">
+    <row r="30" ht="15.75"/>
+    <row r="31" ht="15.75"/>
+    <row r="32" ht="15.75" spans="2:4">
       <c r="B32" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C32" s="57">
         <f>SUM(G17:G29,F9:F13,F4:F5)</f>
@@ -6685,9 +6698,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="2:4">
+    <row r="33" customHeight="1" spans="2:4">
       <c r="B33" s="58" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C33" s="59">
         <f>Clebina!C3*10</f>
@@ -6697,7 +6710,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1" spans="2:4">
       <c r="B34" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C34" s="61" t="str">
         <f>IF(C32&gt;D32,"Sobrecarga","Sem Penalidade")</f>
@@ -6705,7 +6718,7 @@
       </c>
       <c r="D34" s="62"/>
     </row>
-    <row r="35" ht="17.25"/>
+    <row r="35" ht="15.75"/>
   </sheetData>
   <mergeCells count="19">
     <mergeCell ref="B2:F2"/>
@@ -6737,39 +6750,39 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="B1:Q33"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="9.56888888888889" customWidth="1"/>
-    <col min="4" max="4" width="10.5688888888889" customWidth="1"/>
-    <col min="5" max="5" width="13.2844444444444" customWidth="1"/>
-    <col min="6" max="7" width="11.4266666666667" customWidth="1"/>
-    <col min="8" max="8" width="11.1422222222222" customWidth="1"/>
-    <col min="9" max="9" width="21.4266666666667" customWidth="1"/>
-    <col min="10" max="10" width="10.1422222222222" customWidth="1"/>
-    <col min="11" max="11" width="13.8533333333333" customWidth="1"/>
-    <col min="12" max="12" width="21.4266666666667" customWidth="1"/>
-    <col min="13" max="13" width="26.7111111111111" customWidth="1"/>
-    <col min="14" max="14" width="9.85333333333333" customWidth="1"/>
-    <col min="15" max="15" width="12.5688888888889" customWidth="1"/>
+    <col min="3" max="3" width="9.56666666666667" customWidth="1"/>
+    <col min="4" max="4" width="10.5666666666667" customWidth="1"/>
+    <col min="5" max="5" width="13.2833333333333" customWidth="1"/>
+    <col min="6" max="7" width="11.425" customWidth="1"/>
+    <col min="8" max="8" width="11.1416666666667" customWidth="1"/>
+    <col min="9" max="9" width="21.425" customWidth="1"/>
+    <col min="10" max="10" width="10.1416666666667" customWidth="1"/>
+    <col min="11" max="11" width="13.85" customWidth="1"/>
+    <col min="12" max="12" width="21.425" customWidth="1"/>
+    <col min="13" max="13" width="26.7083333333333" customWidth="1"/>
+    <col min="14" max="14" width="9.85" customWidth="1"/>
+    <col min="15" max="15" width="12.5666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25"/>
-    <row r="2" ht="15" customHeight="1" spans="2:16">
+    <row r="1" ht="15.75"/>
+    <row r="2" customHeight="1" spans="2:16">
       <c r="B2" s="24" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>1</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>41</v>
@@ -6778,31 +6791,31 @@
         <v>24</v>
       </c>
       <c r="I2" s="25" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J2" s="25" t="s">
         <v>79</v>
       </c>
       <c r="K2" s="33" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="L2" s="33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M2" s="34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="O2" s="35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P2" s="36"/>
     </row>
     <row r="3" spans="2:16">
       <c r="B3" s="26" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D3" s="27">
         <f>VLOOKUP(C3,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6824,13 +6837,13 @@
         <v>2</v>
       </c>
       <c r="K3" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L3" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M3" s="37" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O3" s="38" t="s">
         <v>34</v>
@@ -6841,10 +6854,10 @@
     </row>
     <row r="4" spans="2:16">
       <c r="B4" s="28" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D4" s="29">
         <f>VLOOKUP(C4,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6866,13 +6879,13 @@
         <v>3</v>
       </c>
       <c r="K4" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L4" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M4" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="M4" s="40" t="s">
-        <v>140</v>
       </c>
       <c r="O4" s="41" t="s">
         <v>57</v>
@@ -6881,12 +6894,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" ht="17.25" spans="2:16">
+    <row r="5" ht="15.75" spans="2:16">
       <c r="B5" s="26" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D5" s="27">
         <f>VLOOKUP(C5,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6908,13 +6921,13 @@
         <v>5</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O5" s="43" t="s">
         <v>71</v>
@@ -6923,12 +6936,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" ht="18" spans="2:13">
+    <row r="6" ht="16.5" spans="2:13">
       <c r="B6" s="28" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D6" s="29">
         <f>VLOOKUP(C6,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6950,21 +6963,21 @@
         <v>3</v>
       </c>
       <c r="K6" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L6" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M6" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" spans="2:16">
       <c r="B7" s="26" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D7" s="27">
         <f>VLOOKUP(C7,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6986,25 +6999,25 @@
         <v>4</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L7" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O7" s="35" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P7" s="36"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="2:16">
+    <row r="8" customHeight="1" spans="2:16">
       <c r="B8" s="28" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D8" s="29">
         <f>VLOOKUP(C8,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7026,13 +7039,13 @@
         <v>10</v>
       </c>
       <c r="K8" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L8" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M8" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L8" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M8" s="40" t="s">
-        <v>140</v>
       </c>
       <c r="O8" s="38" t="s">
         <v>4</v>
@@ -7044,10 +7057,10 @@
     </row>
     <row r="9" spans="2:16">
       <c r="B9" s="26" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D9" s="27">
         <f>VLOOKUP(C9,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7069,13 +7082,13 @@
         <v>8</v>
       </c>
       <c r="K9" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="L9" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="L9" s="27" t="s">
-        <v>140</v>
-      </c>
       <c r="M9" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O9" s="41" t="s">
         <v>9</v>
@@ -7087,10 +7100,10 @@
     </row>
     <row r="10" spans="2:16">
       <c r="B10" s="28" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D10" s="29">
         <f>VLOOKUP(C10,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7112,13 +7125,13 @@
         <v>3</v>
       </c>
       <c r="K10" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L10" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M10" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O10" s="38" t="s">
         <v>10</v>
@@ -7130,10 +7143,10 @@
     </row>
     <row r="11" spans="2:16">
       <c r="B11" s="26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D11" s="27">
         <f>VLOOKUP(C11,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7155,13 +7168,13 @@
         <v>3</v>
       </c>
       <c r="K11" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L11" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O11" s="41" t="s">
         <v>12</v>
@@ -7173,10 +7186,10 @@
     </row>
     <row r="12" spans="2:16">
       <c r="B12" s="28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D12" s="29">
         <f>VLOOKUP(C12,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7198,13 +7211,13 @@
         <v>5</v>
       </c>
       <c r="K12" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L12" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="L12" s="29" t="s">
-        <v>140</v>
-      </c>
       <c r="M12" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O12" s="38" t="s">
         <v>14</v>
@@ -7214,12 +7227,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" ht="17.25" spans="2:16">
+    <row r="13" ht="15.75" spans="2:16">
       <c r="B13" s="26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D13" s="27">
         <f>VLOOKUP(C13,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7241,13 +7254,13 @@
         <v>2</v>
       </c>
       <c r="K13" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L13" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O13" s="45" t="s">
         <v>16</v>
@@ -7257,12 +7270,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="17.25" spans="2:13">
+    <row r="14" ht="15.75" spans="2:13">
       <c r="B14" s="28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D14" s="29">
         <f>VLOOKUP(C14,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7284,21 +7297,21 @@
         <v>10</v>
       </c>
       <c r="K14" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L14" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M14" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L14" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M14" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="15" spans="2:13">
       <c r="B15" s="26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D15" s="27">
         <f>VLOOKUP(C15,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7320,21 +7333,21 @@
         <v>4</v>
       </c>
       <c r="K15" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L15" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="2:13">
       <c r="B16" s="28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D16" s="29">
         <f>VLOOKUP(C16,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7356,21 +7369,21 @@
         <v>3</v>
       </c>
       <c r="K16" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L16" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M16" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="2:17">
       <c r="B17" s="26" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D17" s="27">
         <f>VLOOKUP(C17,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7392,13 +7405,13 @@
         <v>6</v>
       </c>
       <c r="K17" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L17" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q17" t="str">
         <f>IF(P17&gt;P18,"passou demais","")</f>
@@ -7407,10 +7420,10 @@
     </row>
     <row r="18" spans="2:13">
       <c r="B18" s="28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D18" s="29">
         <f>VLOOKUP(C18,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7432,21 +7445,21 @@
         <v>10</v>
       </c>
       <c r="K18" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L18" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="L18" s="29" t="s">
-        <v>140</v>
-      </c>
       <c r="M18" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="2:13">
       <c r="B19" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D19" s="27">
         <f>VLOOKUP(C19,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7468,21 +7481,21 @@
         <v>3</v>
       </c>
       <c r="K19" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L19" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="M19" s="37" t="s">
         <v>141</v>
-      </c>
-      <c r="M19" s="37" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="20" spans="2:13">
       <c r="B20" s="28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D20" s="29">
         <f>VLOOKUP(C20,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7504,13 +7517,13 @@
         <v>2</v>
       </c>
       <c r="K20" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L20" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M20" s="40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" spans="2:13">
@@ -7518,7 +7531,7 @@
         <v>80</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D21" s="27">
         <f>VLOOKUP(C21,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7540,21 +7553,21 @@
         <v>7</v>
       </c>
       <c r="K21" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="L21" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="L21" s="27" t="s">
-        <v>140</v>
-      </c>
       <c r="M21" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="2:13">
       <c r="B22" s="28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D22" s="29">
         <f>VLOOKUP(C22,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7578,21 +7591,21 @@
         <v>12</v>
       </c>
       <c r="K22" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L22" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M22" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L22" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M22" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="23" spans="2:13">
       <c r="B23" s="26" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D23" s="27">
         <f>VLOOKUP(C23,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7614,21 +7627,21 @@
         <v>8</v>
       </c>
       <c r="K23" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L23" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="M23" s="37" t="s">
         <v>141</v>
-      </c>
-      <c r="M23" s="37" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="24" spans="2:13">
       <c r="B24" s="28" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D24" s="29">
         <f>VLOOKUP(C24,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7650,21 +7663,21 @@
         <v>10</v>
       </c>
       <c r="K24" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L24" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M24" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L24" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M24" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="25" spans="2:13">
       <c r="B25" s="26" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D25" s="27">
         <f>VLOOKUP(C25,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7686,21 +7699,21 @@
         <v>10</v>
       </c>
       <c r="K25" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="L25" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="M25" s="37" t="s">
         <v>141</v>
-      </c>
-      <c r="L25" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="M25" s="37" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="26" spans="2:13">
       <c r="B26" s="30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D26" s="29">
         <f>VLOOKUP(C26,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7722,21 +7735,21 @@
         <v>10</v>
       </c>
       <c r="K26" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L26" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M26" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L26" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M26" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="27" spans="2:13">
       <c r="B27" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D27" s="27">
         <f>VLOOKUP(C27,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7760,21 +7773,21 @@
         <v>10</v>
       </c>
       <c r="K27" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="L27" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="L27" s="27" t="s">
-        <v>140</v>
-      </c>
       <c r="M27" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="28" spans="2:13">
       <c r="B28" s="28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D28" s="29">
         <f>VLOOKUP(C28,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7796,21 +7809,21 @@
         <v>4</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L28" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M28" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="M28" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="29" spans="2:13">
       <c r="B29" s="26" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D29" s="27">
         <f>VLOOKUP(C29,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7832,21 +7845,21 @@
         <v>4</v>
       </c>
       <c r="K29" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L29" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M29" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="30" spans="2:13">
       <c r="B30" s="28" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D30" s="29">
         <f>VLOOKUP(C30,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7868,21 +7881,21 @@
         <v>6</v>
       </c>
       <c r="K30" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L30" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="L30" s="29" t="s">
-        <v>140</v>
-      </c>
       <c r="M30" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="2:13">
       <c r="B31" s="26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D31" s="27">
         <f>VLOOKUP(C31,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7904,21 +7917,21 @@
         <v>6</v>
       </c>
       <c r="K31" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L31" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="M31" s="37" t="s">
         <v>141</v>
-      </c>
-      <c r="M31" s="37" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="32" spans="2:13">
       <c r="B32" s="28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D32" s="29">
         <f>VLOOKUP(C32,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7940,21 +7953,21 @@
         <v>6</v>
       </c>
       <c r="K32" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L32" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M32" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33" spans="2:13">
       <c r="B33" s="31" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C33" s="32" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D33" s="32">
         <f>VLOOKUP(C33,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7976,13 +7989,13 @@
         <v>8</v>
       </c>
       <c r="K33" s="32" t="s">
+        <v>142</v>
+      </c>
+      <c r="L33" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="L33" s="32" t="s">
-        <v>140</v>
-      </c>
       <c r="M33" s="47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -8003,39 +8016,39 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="B1:P33"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="9.56888888888889" customWidth="1"/>
-    <col min="4" max="4" width="10.5688888888889" customWidth="1"/>
-    <col min="5" max="5" width="13.2844444444444" customWidth="1"/>
-    <col min="6" max="7" width="11.4266666666667" customWidth="1"/>
-    <col min="8" max="8" width="11.1422222222222" customWidth="1"/>
-    <col min="9" max="9" width="21.4266666666667" customWidth="1"/>
-    <col min="10" max="10" width="10.1422222222222" customWidth="1"/>
-    <col min="11" max="11" width="13.8533333333333" customWidth="1"/>
-    <col min="12" max="12" width="21.4266666666667" customWidth="1"/>
-    <col min="13" max="13" width="26.7111111111111" customWidth="1"/>
-    <col min="14" max="14" width="9.85333333333333" customWidth="1"/>
-    <col min="15" max="15" width="12.5688888888889" customWidth="1"/>
+    <col min="3" max="3" width="9.56666666666667" customWidth="1"/>
+    <col min="4" max="4" width="10.5666666666667" customWidth="1"/>
+    <col min="5" max="5" width="13.2833333333333" customWidth="1"/>
+    <col min="6" max="7" width="11.425" customWidth="1"/>
+    <col min="8" max="8" width="11.1416666666667" customWidth="1"/>
+    <col min="9" max="9" width="21.425" customWidth="1"/>
+    <col min="10" max="10" width="10.1416666666667" customWidth="1"/>
+    <col min="11" max="11" width="13.85" customWidth="1"/>
+    <col min="12" max="12" width="21.425" customWidth="1"/>
+    <col min="13" max="13" width="26.7083333333333" customWidth="1"/>
+    <col min="14" max="14" width="9.85" customWidth="1"/>
+    <col min="15" max="15" width="12.5666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25"/>
-    <row r="2" ht="15" customHeight="1" spans="2:16">
+    <row r="1" ht="15.75"/>
+    <row r="2" customHeight="1" spans="2:16">
       <c r="B2" s="24" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>1</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>41</v>
@@ -8044,31 +8057,31 @@
         <v>24</v>
       </c>
       <c r="I2" s="25" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J2" s="25" t="s">
         <v>79</v>
       </c>
       <c r="K2" s="33" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="L2" s="33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M2" s="34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="O2" s="35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P2" s="36"/>
     </row>
     <row r="3" spans="2:16">
       <c r="B3" s="26" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D3" s="27">
         <f>VLOOKUP(C3,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8090,13 +8103,13 @@
         <v>2</v>
       </c>
       <c r="K3" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L3" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M3" s="37" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O3" s="38" t="s">
         <v>34</v>
@@ -8107,10 +8120,10 @@
     </row>
     <row r="4" spans="2:16">
       <c r="B4" s="28" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D4" s="29">
         <f>VLOOKUP(C4,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8132,13 +8145,13 @@
         <v>3</v>
       </c>
       <c r="K4" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L4" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M4" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="M4" s="40" t="s">
-        <v>140</v>
       </c>
       <c r="O4" s="41" t="s">
         <v>57</v>
@@ -8147,12 +8160,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" ht="17.25" spans="2:16">
+    <row r="5" ht="15.75" spans="2:16">
       <c r="B5" s="26" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D5" s="27">
         <f>VLOOKUP(C5,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8174,13 +8187,13 @@
         <v>5</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O5" s="43" t="s">
         <v>71</v>
@@ -8189,12 +8202,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" ht="18" spans="2:13">
+    <row r="6" ht="16.5" spans="2:13">
       <c r="B6" s="28" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D6" s="29">
         <f>VLOOKUP(C6,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8216,21 +8229,21 @@
         <v>3</v>
       </c>
       <c r="K6" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L6" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M6" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" spans="2:16">
       <c r="B7" s="26" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D7" s="27">
         <f>VLOOKUP(C7,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8252,25 +8265,25 @@
         <v>4</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L7" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O7" s="35" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P7" s="36"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="2:16">
+    <row r="8" customHeight="1" spans="2:16">
       <c r="B8" s="28" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D8" s="29">
         <f>VLOOKUP(C8,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8292,13 +8305,13 @@
         <v>10</v>
       </c>
       <c r="K8" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L8" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M8" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L8" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M8" s="40" t="s">
-        <v>140</v>
       </c>
       <c r="O8" s="38" t="s">
         <v>4</v>
@@ -8310,10 +8323,10 @@
     </row>
     <row r="9" spans="2:16">
       <c r="B9" s="26" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D9" s="27">
         <f>VLOOKUP(C9,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8335,13 +8348,13 @@
         <v>8</v>
       </c>
       <c r="K9" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="L9" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="L9" s="27" t="s">
-        <v>140</v>
-      </c>
       <c r="M9" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O9" s="41" t="s">
         <v>9</v>
@@ -8353,10 +8366,10 @@
     </row>
     <row r="10" spans="2:16">
       <c r="B10" s="28" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D10" s="29">
         <f>VLOOKUP(C10,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8378,13 +8391,13 @@
         <v>3</v>
       </c>
       <c r="K10" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L10" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M10" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O10" s="38" t="s">
         <v>10</v>
@@ -8396,10 +8409,10 @@
     </row>
     <row r="11" spans="2:16">
       <c r="B11" s="26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D11" s="27">
         <f>VLOOKUP(C11,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8421,13 +8434,13 @@
         <v>3</v>
       </c>
       <c r="K11" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L11" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O11" s="41" t="s">
         <v>12</v>
@@ -8439,10 +8452,10 @@
     </row>
     <row r="12" spans="2:16">
       <c r="B12" s="28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D12" s="29">
         <f>VLOOKUP(C12,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8464,13 +8477,13 @@
         <v>3</v>
       </c>
       <c r="K12" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L12" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M12" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O12" s="38" t="s">
         <v>14</v>
@@ -8480,12 +8493,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" ht="17.25" spans="2:16">
+    <row r="13" ht="15.75" spans="2:16">
       <c r="B13" s="26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D13" s="27">
         <f>VLOOKUP(C13,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8507,13 +8520,13 @@
         <v>4</v>
       </c>
       <c r="K13" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L13" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O13" s="45" t="s">
         <v>16</v>
@@ -8523,12 +8536,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="17.25" spans="2:13">
+    <row r="14" ht="15.75" spans="2:13">
       <c r="B14" s="28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D14" s="29">
         <f>VLOOKUP(C14,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8552,21 +8565,21 @@
         <v>11</v>
       </c>
       <c r="K14" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L14" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M14" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L14" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M14" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="15" spans="2:13">
       <c r="B15" s="26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D15" s="27">
         <f>VLOOKUP(C15,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8588,21 +8601,21 @@
         <v>4</v>
       </c>
       <c r="K15" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L15" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="2:13">
       <c r="B16" s="28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D16" s="29">
         <f>VLOOKUP(C16,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8624,21 +8637,21 @@
         <v>3</v>
       </c>
       <c r="K16" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L16" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M16" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="2:13">
       <c r="B17" s="26" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D17" s="27">
         <f>VLOOKUP(C17,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8660,21 +8673,21 @@
         <v>6</v>
       </c>
       <c r="K17" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L17" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="2:13">
       <c r="B18" s="28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D18" s="29">
         <f>VLOOKUP(C18,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8696,21 +8709,21 @@
         <v>10</v>
       </c>
       <c r="K18" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L18" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="L18" s="29" t="s">
-        <v>140</v>
-      </c>
       <c r="M18" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="2:13">
       <c r="B19" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D19" s="27">
         <f>VLOOKUP(C19,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8732,21 +8745,21 @@
         <v>3</v>
       </c>
       <c r="K19" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L19" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="M19" s="37" t="s">
         <v>141</v>
-      </c>
-      <c r="M19" s="37" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="20" spans="2:13">
       <c r="B20" s="28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D20" s="29">
         <f>VLOOKUP(C20,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8768,13 +8781,13 @@
         <v>4</v>
       </c>
       <c r="K20" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L20" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M20" s="40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" spans="2:13">
@@ -8782,7 +8795,7 @@
         <v>80</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D21" s="27">
         <f>VLOOKUP(C21,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8804,21 +8817,21 @@
         <v>7</v>
       </c>
       <c r="K21" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="L21" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="L21" s="27" t="s">
-        <v>140</v>
-      </c>
       <c r="M21" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="2:13">
       <c r="B22" s="28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D22" s="29">
         <f>VLOOKUP(C22,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8842,21 +8855,21 @@
         <v>12</v>
       </c>
       <c r="K22" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L22" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M22" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L22" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M22" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="23" spans="2:13">
       <c r="B23" s="26" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D23" s="27">
         <f>VLOOKUP(C23,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8878,21 +8891,21 @@
         <v>8</v>
       </c>
       <c r="K23" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L23" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="M23" s="37" t="s">
         <v>141</v>
-      </c>
-      <c r="M23" s="37" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="24" spans="2:13">
       <c r="B24" s="28" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D24" s="29">
         <f>VLOOKUP(C24,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8914,21 +8927,21 @@
         <v>10</v>
       </c>
       <c r="K24" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L24" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M24" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L24" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M24" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="25" spans="2:13">
       <c r="B25" s="26" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D25" s="27">
         <f>VLOOKUP(C25,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8950,21 +8963,21 @@
         <v>10</v>
       </c>
       <c r="K25" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="L25" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="M25" s="37" t="s">
         <v>141</v>
-      </c>
-      <c r="L25" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="M25" s="37" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="26" spans="2:13">
       <c r="B26" s="30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D26" s="29">
         <f>VLOOKUP(C26,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8986,21 +8999,21 @@
         <v>10</v>
       </c>
       <c r="K26" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L26" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M26" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="L26" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M26" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="27" spans="2:13">
       <c r="B27" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D27" s="27">
         <f>VLOOKUP(C27,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9024,21 +9037,21 @@
         <v>10</v>
       </c>
       <c r="K27" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="L27" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="L27" s="27" t="s">
-        <v>140</v>
-      </c>
       <c r="M27" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="28" spans="2:13">
       <c r="B28" s="28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D28" s="29">
         <f>VLOOKUP(C28,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9060,21 +9073,21 @@
         <v>4</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L28" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="M28" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="M28" s="40" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="29" spans="2:13">
       <c r="B29" s="26" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D29" s="27">
         <f>VLOOKUP(C29,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9096,21 +9109,21 @@
         <v>4</v>
       </c>
       <c r="K29" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L29" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M29" s="37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="30" spans="2:13">
       <c r="B30" s="28" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D30" s="29">
         <f>VLOOKUP(C30,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9132,21 +9145,21 @@
         <v>6</v>
       </c>
       <c r="K30" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L30" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="L30" s="29" t="s">
-        <v>140</v>
-      </c>
       <c r="M30" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="2:13">
       <c r="B31" s="26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D31" s="27">
         <f>VLOOKUP(C31,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9168,21 +9181,21 @@
         <v>8</v>
       </c>
       <c r="K31" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="L31" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="M31" s="37" t="s">
         <v>141</v>
-      </c>
-      <c r="L31" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="M31" s="37" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="32" spans="2:13">
       <c r="B32" s="28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D32" s="29">
         <f>VLOOKUP(C32,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9204,21 +9217,21 @@
         <v>6</v>
       </c>
       <c r="K32" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L32" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M32" s="40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33" spans="2:13">
       <c r="B33" s="31" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C33" s="32" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D33" s="32">
         <f>VLOOKUP(C33,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9240,13 +9253,13 @@
         <v>8</v>
       </c>
       <c r="K33" s="32" t="s">
+        <v>142</v>
+      </c>
+      <c r="L33" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="L33" s="32" t="s">
-        <v>140</v>
-      </c>
       <c r="M33" s="47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -9267,19 +9280,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="B1:M23"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="3" width="10.2844444444444" customWidth="1"/>
-    <col min="4" max="4" width="12.2844444444444" customWidth="1"/>
-    <col min="8" max="8" width="20.2844444444444" customWidth="1"/>
-    <col min="9" max="9" width="19.8533333333333" customWidth="1"/>
+    <col min="2" max="3" width="10.2833333333333" customWidth="1"/>
+    <col min="4" max="4" width="12.2833333333333" customWidth="1"/>
+    <col min="8" max="8" width="20.2833333333333" customWidth="1"/>
+    <col min="9" max="9" width="19.85" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25"/>
-    <row r="2" ht="17.25" spans="2:13">
+    <row r="1" ht="15.75"/>
+    <row r="2" ht="15.75" spans="2:13">
       <c r="B2" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C2" s="2"/>
       <c r="E2" s="1">
@@ -9289,16 +9302,16 @@
         <v>2</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="M2" s="2">
         <f>12+Clebina!D5</f>
@@ -9329,13 +9342,13 @@
         <v>0</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M3" s="4">
         <v>4</v>
       </c>
     </row>
-    <row r="4" ht="17.25" spans="2:13">
+    <row r="4" ht="15.75" spans="2:13">
       <c r="B4" s="5" t="s">
         <v>9</v>
       </c>
@@ -9359,13 +9372,13 @@
         <v>1</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="M4" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="5" ht="17.25" spans="2:10">
+    <row r="5" ht="15.75" spans="2:10">
       <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
@@ -9419,7 +9432,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" ht="17.25" spans="2:10">
+    <row r="8" ht="15.75" spans="2:10">
       <c r="B8" s="7" t="s">
         <v>16</v>
       </c>
@@ -9437,7 +9450,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" ht="17.25" spans="8:10">
+    <row r="9" ht="15.75" spans="8:10">
       <c r="H9" s="17">
         <v>21000</v>
       </c>
@@ -9461,7 +9474,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" ht="17.25" spans="8:10">
+    <row r="11" ht="15.75" spans="8:10">
       <c r="H11" s="17">
         <v>36000</v>
       </c>
@@ -9473,9 +9486,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" ht="17.25" spans="2:10">
+    <row r="12" ht="15.75" spans="2:10">
       <c r="B12" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C12" s="2">
         <f>3+Clebina!D5</f>
@@ -9494,7 +9507,7 @@
     </row>
     <row r="13" spans="2:10">
       <c r="B13" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C13" s="4">
         <f>SUM(M3:M4)</f>
@@ -9511,7 +9524,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" ht="17.25" spans="2:10">
+    <row r="14" ht="15.75" spans="2:10">
       <c r="B14" s="7"/>
       <c r="C14" s="8"/>
       <c r="H14" s="16">
@@ -9525,7 +9538,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" ht="18" spans="8:10">
+    <row r="15" ht="16.5" spans="8:10">
       <c r="H15" s="17">
         <v>78000</v>
       </c>
@@ -9537,15 +9550,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" ht="17.25" spans="2:10">
+    <row r="16" ht="15.75" spans="2:10">
       <c r="B16" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E16" s="18" t="s">
         <v>79</v>
@@ -9678,7 +9691,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" ht="17.25" spans="2:10">
+    <row r="22" ht="15.75" spans="2:10">
       <c r="B22" s="13" t="s">
         <v>16</v>
       </c>
@@ -9701,7 +9714,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" ht="17.25"/>
+    <row r="23" ht="15.75"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:C2"/>

</xml_diff>

<commit_message>
Upada sessão tormenta 20/07
</commit_message>
<xml_diff>
--- a/Fichas/Tormenta/Ficha Cleber.xlsx
+++ b/Fichas/Tormenta/Ficha Cleber.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7635" activeTab="5"/>
+    <workbookView windowWidth="28800" windowHeight="12315" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Clebina" sheetId="1" r:id="rId1"/>
@@ -152,22 +152,14 @@
       <text>
         <r>
           <rPr>
-            <b/>
             <sz val="9"/>
             <rFont val="Segoe UI"/>
             <charset val="134"/>
           </rPr>
-          <t>Luciano Segundo:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Segoe UI"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
-Invenção Potente - Quando usa um item fabricado por você mesmo, você pode pagar 1 PM para
-aumentar em +2 a CD para resistir a ele.</t>
+          <t>Você recebe proficiência com armas
+marciais corpo a corpo. Quando usa uma arma corpo a corpo, pode usar seu modificador de Inteligência em
+vez de Força nos testes de ataque e rolagens de dano.
+Pré-requisitos: treinado em Luta e Ofício (armeiro).</t>
         </r>
       </text>
     </comment>
@@ -275,10 +267,8 @@
             <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
-Aumento de Atributo. Você recebe +2 em um
-atributo a sua escolha. Você pode escolher este poder
-várias vezes. A partir da segunda vez que escolhê-lo
-para o mesmo atributo, o aumento diminui para +1.</t>
+Invenção Potente - Quando usa um item fabricado por você mesmo, você pode pagar 1 PM para
+aumentar em +2 a CD para resistir a ele.</t>
         </r>
       </text>
     </comment>
@@ -969,7 +959,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="186">
   <si>
     <t>Atributos</t>
   </si>
@@ -1121,39 +1111,36 @@
     <t>Nível 5</t>
   </si>
   <si>
+    <t>Armeiro</t>
+  </si>
+  <si>
+    <t>Origem</t>
+  </si>
+  <si>
+    <t>Venefício</t>
+  </si>
+  <si>
+    <t>Nível 6</t>
+  </si>
+  <si>
+    <t>Alquimista de Batalha</t>
+  </si>
+  <si>
+    <t>Divindade</t>
+  </si>
+  <si>
+    <t>Voz da Civilização</t>
+  </si>
+  <si>
+    <t>Nível 7</t>
+  </si>
+  <si>
     <t>Invenção Potente</t>
   </si>
   <si>
-    <t>Origem</t>
-  </si>
-  <si>
-    <t>Venefício</t>
-  </si>
-  <si>
-    <t>Nível 6</t>
-  </si>
-  <si>
-    <t>Alquimista de Batalha</t>
-  </si>
-  <si>
-    <t>Divindade</t>
-  </si>
-  <si>
-    <t>Voz da Civilização</t>
-  </si>
-  <si>
-    <t>Nível 7</t>
-  </si>
-  <si>
-    <t>Aumento de Atributo</t>
-  </si>
-  <si>
     <t>Nível 8</t>
   </si>
   <si>
-    <t>Armeiro</t>
-  </si>
-  <si>
     <t>Nível 9</t>
   </si>
   <si>
@@ -1263,9 +1250,6 @@
   </si>
   <si>
     <t>Controlar Madeira</t>
-  </si>
-  <si>
-    <t>disc</t>
   </si>
   <si>
     <t>Enxame de Pesteste</t>
@@ -1540,9 +1524,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="179" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="27">
@@ -1581,31 +1565,8 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1627,6 +1588,22 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
@@ -1634,7 +1611,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF9C6500"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1647,9 +1624,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1678,19 +1663,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FF800080"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Aptos Narrow"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1709,16 +1693,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color rgb="FF0000FF"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="Aptos Narrow"/>
       <charset val="134"/>
@@ -1770,7 +1754,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1782,7 +1784,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1794,13 +1796,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1812,7 +1820,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1824,31 +1832,55 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1860,61 +1892,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1926,31 +1922,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2473,6 +2457,30 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -2488,35 +2496,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FF3F3F3F"/>
       </left>
       <right style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FF3F3F3F"/>
       </right>
       <top style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FF3F3F3F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2541,17 +2531,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2573,152 +2557,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="43" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="45" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="41" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="42" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="43" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="45" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="39" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="39" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="40" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="38" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="44" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="44" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="42" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="41" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="41" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="39" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2921,6 +2905,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4341,7 +4326,7 @@
       </c>
       <c r="G2" s="48">
         <f>VLOOKUP(G10,'uns dados aí'!$H$2:$I$22,2,TRUE)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H2" s="36"/>
       <c r="K2" s="35" t="s">
@@ -4368,11 +4353,11 @@
       </c>
       <c r="G3" s="27">
         <f>H3-L25-SUM(L4:L22)</f>
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H3" s="39">
         <f>'uns dados aí'!M2+((G2-1)*'uns dados aí'!C12)</f>
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="K3" s="38" t="s">
         <v>6</v>
@@ -4404,11 +4389,11 @@
       </c>
       <c r="G4" s="29">
         <f>H4-L26-SUM(M4:M22)</f>
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="H4" s="42">
         <f>'uns dados aí'!C13*G2</f>
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="K4" s="41">
         <v>1</v>
@@ -4438,7 +4423,7 @@
         <f>10+D4+C16</f>
         <v>22</v>
       </c>
-      <c r="H5" s="89"/>
+      <c r="H5" s="90"/>
       <c r="K5" s="38">
         <v>2</v>
       </c>
@@ -4467,7 +4452,7 @@
         <f>G5+Perícias!J12</f>
         <v>27</v>
       </c>
-      <c r="H6" s="90"/>
+      <c r="H6" s="91"/>
       <c r="K6" s="41">
         <v>3</v>
       </c>
@@ -4496,7 +4481,7 @@
         <f>Perícias!J27+Perícias!J21</f>
         <v>17</v>
       </c>
-      <c r="H7" s="89"/>
+      <c r="H7" s="90"/>
       <c r="K7" s="38">
         <v>4</v>
       </c>
@@ -4521,10 +4506,10 @@
       <c r="F8" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="91">
+      <c r="G8" s="92">
         <v>0.5</v>
       </c>
-      <c r="H8" s="92"/>
+      <c r="H8" s="93"/>
       <c r="K8" s="41">
         <v>5</v>
       </c>
@@ -4554,7 +4539,7 @@
         <v>19</v>
       </c>
       <c r="G10" s="52">
-        <v>6600</v>
+        <v>10700</v>
       </c>
       <c r="H10" s="46"/>
       <c r="K10" s="41">
@@ -4573,16 +4558,16 @@
       <c r="N11" s="39"/>
     </row>
     <row r="12" ht="16.5" spans="2:14">
-      <c r="B12" s="71" t="s">
+      <c r="B12" s="72" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="72"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="72"/>
-      <c r="F12" s="72"/>
-      <c r="G12" s="72"/>
-      <c r="H12" s="72"/>
-      <c r="I12" s="73"/>
+      <c r="C12" s="73"/>
+      <c r="D12" s="73"/>
+      <c r="E12" s="73"/>
+      <c r="F12" s="73"/>
+      <c r="G12" s="73"/>
+      <c r="H12" s="73"/>
+      <c r="I12" s="74"/>
       <c r="K12" s="41">
         <v>9</v>
       </c>
@@ -4591,7 +4576,7 @@
       <c r="N12" s="42"/>
     </row>
     <row r="13" ht="15.75" spans="2:14">
-      <c r="B13" s="88"/>
+      <c r="B13" s="89"/>
       <c r="K13" s="38">
         <v>10</v>
       </c>
@@ -4782,7 +4767,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="12" max="12" width="19.7083333333333" customWidth="1"/>
@@ -4791,24 +4776,24 @@
   </cols>
   <sheetData>
     <row r="1" ht="16.5" spans="1:15">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="72" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="73"/>
-      <c r="I1" s="71" t="s">
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="74"/>
+      <c r="I1" s="72" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="74"/>
     </row>
     <row r="2" ht="15"/>
     <row r="3" ht="15.75" spans="2:13">
@@ -4821,13 +4806,13 @@
       </c>
       <c r="E3" s="48"/>
       <c r="F3" s="36"/>
-      <c r="K3" s="75" t="s">
+      <c r="K3" s="76" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="76" t="s">
+      <c r="L3" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="M3" s="84" t="s">
+      <c r="M3" s="85" t="s">
         <v>24</v>
       </c>
     </row>
@@ -4843,13 +4828,13 @@
       <c r="F4" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="77" t="s">
+      <c r="K4" s="78" t="s">
         <v>41</v>
       </c>
-      <c r="L4" s="78" t="s">
+      <c r="L4" s="79" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="85"/>
+      <c r="M4" s="86"/>
     </row>
     <row r="5" ht="15" customHeight="1" spans="2:13">
       <c r="B5" s="41" t="s">
@@ -4863,13 +4848,13 @@
       <c r="F5" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="K5" s="79" t="s">
+      <c r="K5" s="80" t="s">
         <v>41</v>
       </c>
-      <c r="L5" s="80" t="s">
+      <c r="L5" s="81" t="s">
         <v>45</v>
       </c>
-      <c r="M5" s="86"/>
+      <c r="M5" s="87"/>
     </row>
     <row r="6" ht="15" customHeight="1" spans="2:13">
       <c r="B6" s="38" t="s">
@@ -4883,13 +4868,13 @@
       <c r="F6" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K6" s="77" t="s">
+      <c r="K6" s="78" t="s">
         <v>41</v>
       </c>
-      <c r="L6" s="78" t="s">
+      <c r="L6" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="M6" s="85"/>
+      <c r="M6" s="86"/>
     </row>
     <row r="7" ht="15" spans="2:13">
       <c r="B7" s="41" t="s">
@@ -4903,13 +4888,13 @@
       <c r="F7" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="K7" s="79" t="s">
+      <c r="K7" s="80" t="s">
         <v>51</v>
       </c>
-      <c r="L7" s="80" t="s">
+      <c r="L7" s="81" t="s">
         <v>52</v>
       </c>
-      <c r="M7" s="86"/>
+      <c r="M7" s="87"/>
     </row>
     <row r="8" ht="14.25" spans="2:13">
       <c r="B8" s="38" t="s">
@@ -4923,13 +4908,13 @@
       <c r="F8" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K8" s="77" t="s">
+      <c r="K8" s="78" t="s">
         <v>55</v>
       </c>
-      <c r="L8" s="81" t="s">
+      <c r="L8" s="82" t="s">
         <v>56</v>
       </c>
-      <c r="M8" s="85"/>
+      <c r="M8" s="86"/>
     </row>
     <row r="9" ht="15" spans="2:13">
       <c r="B9" s="41" t="s">
@@ -4943,9 +4928,9 @@
       <c r="F9" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="79"/>
-      <c r="L9" s="80"/>
-      <c r="M9" s="86"/>
+      <c r="K9" s="80"/>
+      <c r="L9" s="81"/>
+      <c r="M9" s="87"/>
     </row>
     <row r="10" ht="15" customHeight="1" spans="2:13">
       <c r="B10" s="38" t="s">
@@ -4953,174 +4938,173 @@
       </c>
       <c r="C10" s="27"/>
       <c r="D10" s="27" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K10" s="77"/>
-      <c r="L10" s="78"/>
-      <c r="M10" s="85"/>
+      <c r="K10" s="78"/>
+      <c r="L10" s="79"/>
+      <c r="M10" s="86"/>
     </row>
     <row r="11" ht="15" spans="2:13">
       <c r="B11" s="41" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C11" s="29"/>
       <c r="D11" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E11" s="29"/>
       <c r="F11" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="79"/>
-      <c r="L11" s="80"/>
-      <c r="M11" s="86"/>
+      <c r="K11" s="80"/>
+      <c r="L11" s="81"/>
+      <c r="M11" s="87"/>
     </row>
     <row r="12" ht="14.25" spans="2:13">
       <c r="B12" s="38" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C12" s="27"/>
       <c r="D12" s="27" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E12" s="27"/>
       <c r="F12" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="K12" s="77"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="85"/>
+      <c r="K12" s="78"/>
+      <c r="L12" s="79"/>
+      <c r="M12" s="86"/>
     </row>
     <row r="13" ht="15" spans="2:13">
       <c r="B13" s="41" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C13" s="29"/>
       <c r="D13" s="29" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E13" s="29"/>
       <c r="F13" s="42" t="s">
-        <v>67</v>
-      </c>
-      <c r="G13" s="74"/>
-      <c r="K13" s="79"/>
-      <c r="L13" s="80"/>
-      <c r="M13" s="86"/>
+        <v>66</v>
+      </c>
+      <c r="G13" s="75"/>
+      <c r="K13" s="80"/>
+      <c r="L13" s="81"/>
+      <c r="M13" s="87"/>
     </row>
     <row r="14" ht="14.25" spans="2:13">
       <c r="B14" s="38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C14" s="27"/>
       <c r="D14" s="27"/>
       <c r="E14" s="27"/>
       <c r="F14" s="39"/>
-      <c r="K14" s="77"/>
-      <c r="L14" s="78"/>
-      <c r="M14" s="85"/>
+      <c r="K14" s="78"/>
+      <c r="L14" s="79"/>
+      <c r="M14" s="86"/>
     </row>
     <row r="15" ht="15" spans="2:13">
       <c r="B15" s="41" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C15" s="29"/>
       <c r="D15" s="29"/>
       <c r="E15" s="29"/>
       <c r="F15" s="42"/>
-      <c r="K15" s="79"/>
-      <c r="L15" s="80"/>
-      <c r="M15" s="86"/>
+      <c r="K15" s="80"/>
+      <c r="L15" s="81"/>
+      <c r="M15" s="87"/>
     </row>
     <row r="16" ht="14.25" spans="2:13">
       <c r="B16" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C16" s="27"/>
       <c r="D16" s="27"/>
       <c r="E16" s="27"/>
       <c r="F16" s="39"/>
-      <c r="K16" s="77"/>
-      <c r="L16" s="78"/>
-      <c r="M16" s="85"/>
+      <c r="K16" s="78"/>
+      <c r="L16" s="79"/>
+      <c r="M16" s="86"/>
     </row>
     <row r="17" ht="15" spans="2:13">
       <c r="B17" s="41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C17" s="29"/>
       <c r="D17" s="29"/>
       <c r="E17" s="29"/>
       <c r="F17" s="42"/>
-      <c r="K17" s="79"/>
-      <c r="L17" s="80"/>
-      <c r="M17" s="86"/>
+      <c r="K17" s="80"/>
+      <c r="L17" s="81"/>
+      <c r="M17" s="87"/>
     </row>
     <row r="18" ht="14.25" spans="2:13">
       <c r="B18" s="38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C18" s="27"/>
       <c r="D18" s="27"/>
       <c r="E18" s="27"/>
       <c r="F18" s="39"/>
-      <c r="K18" s="77"/>
-      <c r="L18" s="78"/>
-      <c r="M18" s="85"/>
+      <c r="K18" s="78"/>
+      <c r="L18" s="79"/>
+      <c r="M18" s="86"/>
     </row>
     <row r="19" ht="15" spans="2:13">
       <c r="B19" s="41" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C19" s="29"/>
       <c r="D19" s="29"/>
       <c r="E19" s="29"/>
       <c r="F19" s="42"/>
-      <c r="K19" s="79"/>
-      <c r="L19" s="80"/>
-      <c r="M19" s="86"/>
+      <c r="K19" s="80"/>
+      <c r="L19" s="81"/>
+      <c r="M19" s="87"/>
     </row>
     <row r="20" ht="14.25" spans="2:13">
       <c r="B20" s="38" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C20" s="27"/>
       <c r="D20" s="27"/>
       <c r="E20" s="27"/>
       <c r="F20" s="39"/>
-      <c r="K20" s="77"/>
-      <c r="L20" s="78"/>
-      <c r="M20" s="85"/>
+      <c r="K20" s="78"/>
+      <c r="L20" s="79"/>
+      <c r="M20" s="86"/>
     </row>
     <row r="21" ht="15" spans="2:13">
       <c r="B21" s="41" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C21" s="29"/>
       <c r="D21" s="29"/>
       <c r="E21" s="29"/>
       <c r="F21" s="42"/>
-      <c r="K21" s="79"/>
-      <c r="L21" s="80"/>
-      <c r="M21" s="86"/>
+      <c r="K21" s="80"/>
+      <c r="L21" s="81"/>
+      <c r="M21" s="87"/>
     </row>
     <row r="22" ht="15" spans="2:13">
       <c r="B22" s="43" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" s="49"/>
       <c r="D22" s="49"/>
       <c r="E22" s="49"/>
       <c r="F22" s="44"/>
-      <c r="K22" s="82"/>
-      <c r="L22" s="83"/>
-      <c r="M22" s="87"/>
-    </row>
-    <row r="23" ht="14.25"/>
+      <c r="K22" s="83"/>
+      <c r="L22" s="84"/>
+      <c r="M22" s="88"/>
+    </row>
   </sheetData>
   <mergeCells count="42">
     <mergeCell ref="A1:G1"/>
@@ -5188,16 +5172,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="48" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="E2" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="36" t="s">
-        <v>79</v>
-      </c>
       <c r="G2" s="50" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H2" s="64"/>
     </row>
@@ -5212,18 +5196,18 @@
       </c>
       <c r="D3" s="27">
         <f ca="1">RANDBETWEEN(1,20)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E3" s="39">
         <f ca="1">SUM(C3:D3)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G3" s="43" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H3" s="44">
         <f ca="1">VLOOKUP(G3,B2:E31,4,FALSE)</f>
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" ht="15.75" spans="2:5">
@@ -5237,11 +5221,11 @@
       </c>
       <c r="D4" s="29">
         <f ca="1" t="shared" ref="D4:D31" si="0">RANDBETWEEN(1,20)</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E4" s="42">
         <f ca="1" t="shared" ref="E4:E31" si="1">SUM(C4:D4)</f>
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" ht="14.25" spans="2:5">
@@ -5255,11 +5239,11 @@
       </c>
       <c r="D5" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E5" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" ht="15" spans="2:5">
@@ -5273,11 +5257,11 @@
       </c>
       <c r="D6" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E6" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" ht="14.25" spans="2:5">
@@ -5291,11 +5275,11 @@
       </c>
       <c r="D7" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" ht="15" spans="2:5">
@@ -5309,11 +5293,11 @@
       </c>
       <c r="D8" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E8" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" ht="14.25" spans="2:5">
@@ -5327,11 +5311,11 @@
       </c>
       <c r="D9" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E9" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" ht="15" spans="2:5">
@@ -5345,11 +5329,11 @@
       </c>
       <c r="D10" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E10" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" ht="14.25" spans="2:5">
@@ -5363,11 +5347,11 @@
       </c>
       <c r="D11" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E11" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" ht="15" spans="2:5">
@@ -5381,11 +5365,11 @@
       </c>
       <c r="D12" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E12" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" ht="14.25" spans="2:5">
@@ -5399,11 +5383,11 @@
       </c>
       <c r="D13" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E13" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" ht="15" spans="2:5">
@@ -5417,11 +5401,11 @@
       </c>
       <c r="D14" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E14" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" ht="14.25" spans="2:5">
@@ -5435,11 +5419,11 @@
       </c>
       <c r="D15" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E15" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" ht="15" spans="2:5">
@@ -5453,11 +5437,11 @@
       </c>
       <c r="D16" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E16" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" ht="14.25" spans="2:5">
@@ -5471,11 +5455,11 @@
       </c>
       <c r="D17" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E17" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" ht="15" spans="2:5">
@@ -5489,11 +5473,11 @@
       </c>
       <c r="D18" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E18" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" ht="14.25" spans="2:5">
@@ -5507,11 +5491,11 @@
       </c>
       <c r="D19" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E19" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" ht="15" spans="2:5">
@@ -5525,11 +5509,11 @@
       </c>
       <c r="D20" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E20" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" ht="14.25" spans="2:5">
@@ -5543,11 +5527,11 @@
       </c>
       <c r="D21" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E21" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" ht="15" spans="2:5">
@@ -5561,11 +5545,11 @@
       </c>
       <c r="D22" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E22" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" ht="14.25" spans="2:5">
@@ -5579,11 +5563,11 @@
       </c>
       <c r="D23" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E23" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" ht="30" spans="2:5">
@@ -5597,11 +5581,11 @@
       </c>
       <c r="D24" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E24" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" ht="14.25" spans="2:5">
@@ -5615,11 +5599,11 @@
       </c>
       <c r="D25" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E25" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" ht="30" spans="2:5">
@@ -5633,11 +5617,11 @@
       </c>
       <c r="D26" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E26" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" ht="14.25" spans="2:5">
@@ -5651,11 +5635,11 @@
       </c>
       <c r="D27" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E27" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" ht="15" spans="2:5">
@@ -5669,11 +5653,11 @@
       </c>
       <c r="D28" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E28" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" ht="14.25" spans="2:5">
@@ -5687,11 +5671,11 @@
       </c>
       <c r="D29" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E29" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="30" ht="15" spans="2:5">
@@ -5705,11 +5689,11 @@
       </c>
       <c r="D30" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E30" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" ht="15" spans="2:5">
@@ -5723,11 +5707,11 @@
       </c>
       <c r="D31" s="49">
         <f ca="1" t="shared" si="0"/>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E31" s="44">
         <f ca="1" t="shared" si="1"/>
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" ht="14.25"/>
@@ -5760,28 +5744,28 @@
     <row r="1" ht="14.25"/>
     <row r="2" ht="15.75" spans="2:8">
       <c r="B2" s="24" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>36</v>
       </c>
       <c r="D2" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="71" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="70" t="s">
+      <c r="G2" s="35" t="s">
         <v>83</v>
-      </c>
-      <c r="G2" s="35" t="s">
-        <v>84</v>
       </c>
       <c r="H2" s="36"/>
     </row>
     <row r="3" ht="14.25" spans="2:8">
       <c r="B3" s="67" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="67" t="s">
         <v>85</v>
-      </c>
-      <c r="C3" s="67" t="s">
-        <v>86</v>
       </c>
       <c r="D3" s="27">
         <v>1</v>
@@ -5799,10 +5783,10 @@
     </row>
     <row r="4" ht="15" spans="2:8">
       <c r="B4" s="30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D4" s="29">
         <v>1</v>
@@ -5820,10 +5804,10 @@
     </row>
     <row r="5" ht="14.25" spans="2:8">
       <c r="B5" s="67" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" s="26" t="s">
         <v>88</v>
-      </c>
-      <c r="C5" s="26" t="s">
-        <v>89</v>
       </c>
       <c r="D5" s="27">
         <v>1</v>
@@ -5841,10 +5825,10 @@
     </row>
     <row r="6" ht="15" spans="2:8">
       <c r="B6" s="30" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D6" s="29">
         <v>1</v>
@@ -5863,10 +5847,10 @@
     <row r="7" ht="15" spans="1:8">
       <c r="A7" s="68"/>
       <c r="B7" s="67" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D7" s="27">
         <v>1</v>
@@ -5885,10 +5869,10 @@
     </row>
     <row r="8" ht="15.75" spans="2:5">
       <c r="B8" s="30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D8" s="29">
         <v>1</v>
@@ -5898,12 +5882,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="14.25" spans="2:5">
+    <row r="9" ht="14.25" spans="1:6">
+      <c r="A9" s="69"/>
       <c r="B9" s="67" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D9" s="27">
         <v>1</v>
@@ -5912,13 +5897,14 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
+      <c r="F9" s="69"/>
     </row>
     <row r="10" ht="15" spans="2:5">
       <c r="B10" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D10" s="29">
         <v>1</v>
@@ -5930,10 +5916,10 @@
     </row>
     <row r="11" ht="14.25" spans="2:5">
       <c r="B11" s="67" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D11" s="27">
         <v>2</v>
@@ -5945,10 +5931,10 @@
     </row>
     <row r="12" ht="15" spans="2:5">
       <c r="B12" s="30" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D12" s="29">
         <v>1</v>
@@ -5958,12 +5944,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" ht="14.25" spans="2:7">
+    <row r="13" ht="14.25" spans="2:5">
       <c r="B13" s="67" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D13" s="27">
         <v>2</v>
@@ -5972,16 +5958,13 @@
         <f t="shared" si="0"/>
         <v>90</v>
       </c>
-      <c r="G13" t="s">
-        <v>98</v>
-      </c>
     </row>
     <row r="14" ht="15" spans="2:5">
       <c r="B14" s="30" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C14" s="28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D14" s="29">
         <v>2</v>
@@ -5993,10 +5976,10 @@
     </row>
     <row r="15" ht="14.25" spans="2:5">
       <c r="B15" s="67" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D15" s="27">
         <v>2</v>
@@ -6008,10 +5991,10 @@
     </row>
     <row r="16" ht="15" spans="2:5">
       <c r="B16" s="30" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D16" s="29">
         <v>3</v>
@@ -6184,7 +6167,7 @@
       </c>
     </row>
     <row r="35" ht="14.25" spans="2:5">
-      <c r="B35" s="69"/>
+      <c r="B35" s="70"/>
       <c r="C35" s="31"/>
       <c r="D35" s="32"/>
       <c r="E35" s="47" t="str">
@@ -6219,7 +6202,7 @@
     <row r="1" ht="14.25"/>
     <row r="2" ht="15.75" spans="2:6">
       <c r="B2" s="35" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C2" s="48"/>
       <c r="D2" s="48"/>
@@ -6237,10 +6220,10 @@
         <v>25</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F3" s="39" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" ht="15" spans="2:6">
@@ -6270,7 +6253,7 @@
     <row r="6" ht="15"/>
     <row r="7" ht="15.75" spans="2:8">
       <c r="B7" s="50" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C7" s="51"/>
       <c r="D7" s="51"/>
@@ -6287,13 +6270,13 @@
         <v>26</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E8" s="27" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G8" s="37" t="s">
         <v>36</v>
@@ -6307,37 +6290,37 @@
         <v>30</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D9" s="29"/>
       <c r="E9" s="29"/>
       <c r="F9" s="40"/>
       <c r="G9" s="40" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H9" s="42" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" ht="14.25" spans="2:8">
       <c r="B10" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="C10" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="27" t="s">
         <v>111</v>
-      </c>
-      <c r="C10" s="27" t="s">
-        <v>112</v>
-      </c>
-      <c r="D10" s="27" t="s">
-        <v>113</v>
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="37">
         <v>2</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H10" s="39" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" ht="15" spans="2:8">
@@ -6370,7 +6353,7 @@
     <row r="14" ht="15"/>
     <row r="15" ht="15.75" spans="2:9">
       <c r="B15" s="35" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C15" s="48"/>
       <c r="D15" s="48"/>
@@ -6389,27 +6372,27 @@
       </c>
       <c r="D16" s="54"/>
       <c r="E16" s="54" t="s">
+        <v>113</v>
+      </c>
+      <c r="F16" s="54" t="s">
+        <v>114</v>
+      </c>
+      <c r="G16" s="54" t="s">
+        <v>103</v>
+      </c>
+      <c r="H16" s="54" t="s">
         <v>115</v>
       </c>
-      <c r="F16" s="54" t="s">
-        <v>116</v>
-      </c>
-      <c r="G16" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="H16" s="54" t="s">
-        <v>117</v>
-      </c>
       <c r="I16" s="66" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" ht="15" spans="2:9">
       <c r="B17" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="C17" s="93" t="s">
-        <v>119</v>
+        <v>116</v>
+      </c>
+      <c r="C17" s="94" t="s">
+        <v>117</v>
       </c>
       <c r="D17" s="11"/>
       <c r="E17" s="29">
@@ -6432,10 +6415,10 @@
     </row>
     <row r="18" ht="14.25" spans="2:9">
       <c r="B18" s="53" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C18" s="54" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D18" s="54"/>
       <c r="E18" s="54">
@@ -6456,10 +6439,10 @@
     </row>
     <row r="19" ht="15" spans="2:9">
       <c r="B19" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="29">
@@ -6480,7 +6463,7 @@
     </row>
     <row r="20" ht="14.25" spans="2:9">
       <c r="B20" s="53" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C20" s="54"/>
       <c r="D20" s="54"/>
@@ -6502,7 +6485,7 @@
     </row>
     <row r="21" ht="15" spans="2:9">
       <c r="B21" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
@@ -6602,7 +6585,7 @@
     <row r="31" ht="14.25"/>
     <row r="32" ht="15.75" spans="2:4">
       <c r="B32" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C32" s="56">
         <f>SUM(G17:G29,F9:F13,F4:F5)</f>
@@ -6615,7 +6598,7 @@
     </row>
     <row r="33" ht="15" customHeight="1" spans="2:4">
       <c r="B33" s="57" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C33" s="58">
         <f>Clebina!C3*10</f>
@@ -6625,7 +6608,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1" spans="2:4">
       <c r="B34" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C34" s="60" t="str">
         <f>IF(C32&gt;D32,"Sobrecarga","Sem Penalidade")</f>
@@ -6685,19 +6668,19 @@
     <row r="1" ht="14.25"/>
     <row r="2" ht="15" customHeight="1" spans="2:16">
       <c r="B2" s="24" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>1</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>41</v>
@@ -6706,31 +6689,31 @@
         <v>24</v>
       </c>
       <c r="I2" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="K2" s="33" t="s">
+        <v>131</v>
+      </c>
+      <c r="L2" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="J2" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="K2" s="33" t="s">
+      <c r="M2" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="L2" s="33" t="s">
+      <c r="O2" s="35" t="s">
         <v>134</v>
-      </c>
-      <c r="M2" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="O2" s="35" t="s">
-        <v>136</v>
       </c>
       <c r="P2" s="36"/>
     </row>
     <row r="3" ht="14.25" spans="2:16">
       <c r="B3" s="26" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D3" s="27">
         <f>VLOOKUP(C3,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6752,13 +6735,13 @@
         <v>2</v>
       </c>
       <c r="K3" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="L3" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="M3" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="L3" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="M3" s="37" t="s">
-        <v>141</v>
       </c>
       <c r="O3" s="38" t="s">
         <v>34</v>
@@ -6769,10 +6752,10 @@
     </row>
     <row r="4" ht="15" spans="2:16">
       <c r="B4" s="28" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D4" s="29">
         <f>VLOOKUP(C4,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6794,13 +6777,13 @@
         <v>3</v>
       </c>
       <c r="K4" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="L4" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L4" s="29" t="s">
-        <v>141</v>
-      </c>
       <c r="M4" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O4" s="41" t="s">
         <v>57</v>
@@ -6811,10 +6794,10 @@
     </row>
     <row r="5" ht="15" spans="2:16">
       <c r="B5" s="26" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D5" s="27">
         <f>VLOOKUP(C5,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6836,16 +6819,16 @@
         <v>5</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O5" s="43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P5" s="44">
         <v>6</v>
@@ -6853,10 +6836,10 @@
     </row>
     <row r="6" ht="16.5" spans="2:13">
       <c r="B6" s="28" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D6" s="29">
         <f>VLOOKUP(C6,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6878,21 +6861,21 @@
         <v>3</v>
       </c>
       <c r="K6" s="29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L6" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M6" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" spans="2:16">
       <c r="B7" s="26" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D7" s="27">
         <f>VLOOKUP(C7,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6914,25 +6897,25 @@
         <v>4</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L7" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O7" s="35" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="P7" s="36"/>
     </row>
     <row r="8" ht="15" customHeight="1" spans="2:16">
       <c r="B8" s="28" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D8" s="29">
         <f>VLOOKUP(C8,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6954,13 +6937,13 @@
         <v>10</v>
       </c>
       <c r="K8" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L8" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M8" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O8" s="38" t="s">
         <v>4</v>
@@ -6972,10 +6955,10 @@
     </row>
     <row r="9" ht="15" spans="2:16">
       <c r="B9" s="26" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D9" s="27">
         <f>VLOOKUP(C9,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -6997,13 +6980,13 @@
         <v>8</v>
       </c>
       <c r="K9" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L9" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M9" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O9" s="41" t="s">
         <v>9</v>
@@ -7015,10 +6998,10 @@
     </row>
     <row r="10" ht="15" spans="2:16">
       <c r="B10" s="28" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D10" s="29">
         <f>VLOOKUP(C10,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7040,13 +7023,13 @@
         <v>3</v>
       </c>
       <c r="K10" s="29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L10" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M10" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O10" s="38" t="s">
         <v>10</v>
@@ -7058,10 +7041,10 @@
     </row>
     <row r="11" ht="15" spans="2:16">
       <c r="B11" s="26" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D11" s="27">
         <f>VLOOKUP(C11,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7083,13 +7066,13 @@
         <v>3</v>
       </c>
       <c r="K11" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L11" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O11" s="41" t="s">
         <v>12</v>
@@ -7101,10 +7084,10 @@
     </row>
     <row r="12" ht="15" spans="2:16">
       <c r="B12" s="28" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D12" s="29">
         <f>VLOOKUP(C12,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7126,13 +7109,13 @@
         <v>5</v>
       </c>
       <c r="K12" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L12" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M12" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O12" s="38" t="s">
         <v>14</v>
@@ -7144,10 +7127,10 @@
     </row>
     <row r="13" ht="15.75" spans="2:16">
       <c r="B13" s="26" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D13" s="27">
         <f>VLOOKUP(C13,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7169,13 +7152,13 @@
         <v>2</v>
       </c>
       <c r="K13" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="L13" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="M13" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="L13" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="M13" s="37" t="s">
-        <v>141</v>
       </c>
       <c r="O13" s="45" t="s">
         <v>16</v>
@@ -7187,10 +7170,10 @@
     </row>
     <row r="14" ht="15.75" spans="2:13">
       <c r="B14" s="28" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D14" s="29">
         <f>VLOOKUP(C14,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7212,21 +7195,21 @@
         <v>10</v>
       </c>
       <c r="K14" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L14" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M14" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" ht="14.25" spans="2:13">
       <c r="B15" s="26" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D15" s="27">
         <f>VLOOKUP(C15,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7248,21 +7231,21 @@
         <v>4</v>
       </c>
       <c r="K15" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L15" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" ht="15" spans="2:13">
       <c r="B16" s="28" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D16" s="29">
         <f>VLOOKUP(C16,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7284,21 +7267,21 @@
         <v>3</v>
       </c>
       <c r="K16" s="29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L16" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M16" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" ht="14.25" spans="2:17">
       <c r="B17" s="26" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D17" s="27">
         <f>VLOOKUP(C17,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7320,13 +7303,13 @@
         <v>6</v>
       </c>
       <c r="K17" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L17" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="Q17" t="str">
         <f>IF(P17&gt;P18,"passou demais","")</f>
@@ -7335,10 +7318,10 @@
     </row>
     <row r="18" ht="15" spans="2:13">
       <c r="B18" s="28" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D18" s="29">
         <f>VLOOKUP(C18,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7360,21 +7343,21 @@
         <v>10</v>
       </c>
       <c r="K18" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L18" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M18" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" ht="14.25" spans="2:13">
       <c r="B19" s="26" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D19" s="27">
         <f>VLOOKUP(C19,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7396,21 +7379,21 @@
         <v>3</v>
       </c>
       <c r="K19" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="L19" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L19" s="27" t="s">
-        <v>141</v>
-      </c>
       <c r="M19" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" ht="15" spans="2:13">
       <c r="B20" s="28" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D20" s="29">
         <f>VLOOKUP(C20,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7432,21 +7415,21 @@
         <v>2</v>
       </c>
       <c r="K20" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="L20" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L20" s="29" t="s">
-        <v>141</v>
-      </c>
       <c r="M20" s="40" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" ht="14.25" spans="2:13">
       <c r="B21" s="26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D21" s="27">
         <f>VLOOKUP(C21,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7468,21 +7451,21 @@
         <v>7</v>
       </c>
       <c r="K21" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L21" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M21" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" ht="15" spans="2:13">
       <c r="B22" s="28" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D22" s="29">
         <f>VLOOKUP(C22,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7506,21 +7489,21 @@
         <v>12</v>
       </c>
       <c r="K22" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L22" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M22" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23" ht="14.25" spans="2:13">
       <c r="B23" s="26" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D23" s="27">
         <f>VLOOKUP(C23,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7542,21 +7525,21 @@
         <v>8</v>
       </c>
       <c r="K23" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="L23" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L23" s="27" t="s">
-        <v>141</v>
-      </c>
       <c r="M23" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" ht="15" spans="2:13">
       <c r="B24" s="28" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D24" s="29">
         <f>VLOOKUP(C24,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7578,21 +7561,21 @@
         <v>10</v>
       </c>
       <c r="K24" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L24" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M24" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" ht="14.25" spans="2:13">
       <c r="B25" s="26" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D25" s="27">
         <f>VLOOKUP(C25,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7614,21 +7597,21 @@
         <v>10</v>
       </c>
       <c r="K25" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L25" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M25" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" ht="15" spans="2:13">
       <c r="B26" s="30" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D26" s="29">
         <f>VLOOKUP(C26,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7650,21 +7633,21 @@
         <v>10</v>
       </c>
       <c r="K26" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L26" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M26" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="27" ht="14.25" spans="2:13">
       <c r="B27" s="26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D27" s="27">
         <f>VLOOKUP(C27,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7688,21 +7671,21 @@
         <v>10</v>
       </c>
       <c r="K27" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L27" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M27" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="28" ht="15" spans="2:13">
       <c r="B28" s="28" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D28" s="29">
         <f>VLOOKUP(C28,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7724,21 +7707,21 @@
         <v>4</v>
       </c>
       <c r="K28" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="L28" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L28" s="29" t="s">
-        <v>141</v>
-      </c>
       <c r="M28" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" ht="14.25" spans="2:13">
       <c r="B29" s="26" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D29" s="27">
         <f>VLOOKUP(C29,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7760,21 +7743,21 @@
         <v>4</v>
       </c>
       <c r="K29" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L29" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M29" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30" ht="15" spans="2:13">
       <c r="B30" s="28" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D30" s="29">
         <f>VLOOKUP(C30,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7796,21 +7779,21 @@
         <v>6</v>
       </c>
       <c r="K30" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L30" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M30" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" ht="14.25" spans="2:13">
       <c r="B31" s="26" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D31" s="27">
         <f>VLOOKUP(C31,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7832,21 +7815,21 @@
         <v>6</v>
       </c>
       <c r="K31" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="L31" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L31" s="27" t="s">
-        <v>141</v>
-      </c>
       <c r="M31" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" ht="15" spans="2:13">
       <c r="B32" s="28" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D32" s="29">
         <f>VLOOKUP(C32,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7868,21 +7851,21 @@
         <v>6</v>
       </c>
       <c r="K32" s="29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L32" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M32" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="33" ht="14.25" spans="2:13">
       <c r="B33" s="31" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C33" s="32" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D33" s="32">
         <f>VLOOKUP(C33,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -7904,13 +7887,13 @@
         <v>8</v>
       </c>
       <c r="K33" s="32" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L33" s="32" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M33" s="47" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -7951,19 +7934,19 @@
     <row r="1" ht="14.25"/>
     <row r="2" ht="15" customHeight="1" spans="2:16">
       <c r="B2" s="24" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>1</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>41</v>
@@ -7972,31 +7955,31 @@
         <v>24</v>
       </c>
       <c r="I2" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="K2" s="33" t="s">
+        <v>131</v>
+      </c>
+      <c r="L2" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="J2" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="K2" s="33" t="s">
+      <c r="M2" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="L2" s="33" t="s">
+      <c r="O2" s="35" t="s">
         <v>134</v>
-      </c>
-      <c r="M2" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="O2" s="35" t="s">
-        <v>136</v>
       </c>
       <c r="P2" s="36"/>
     </row>
     <row r="3" ht="14.25" spans="2:16">
       <c r="B3" s="26" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D3" s="27">
         <f>VLOOKUP(C3,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8018,13 +8001,13 @@
         <v>2</v>
       </c>
       <c r="K3" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="L3" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="M3" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="L3" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="M3" s="37" t="s">
-        <v>141</v>
       </c>
       <c r="O3" s="38" t="s">
         <v>34</v>
@@ -8035,10 +8018,10 @@
     </row>
     <row r="4" ht="15" spans="2:16">
       <c r="B4" s="28" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D4" s="29">
         <f>VLOOKUP(C4,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8060,13 +8043,13 @@
         <v>3</v>
       </c>
       <c r="K4" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="L4" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L4" s="29" t="s">
-        <v>141</v>
-      </c>
       <c r="M4" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O4" s="41" t="s">
         <v>57</v>
@@ -8077,10 +8060,10 @@
     </row>
     <row r="5" ht="15" spans="2:16">
       <c r="B5" s="26" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D5" s="27">
         <f>VLOOKUP(C5,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8102,16 +8085,16 @@
         <v>5</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O5" s="43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P5" s="44">
         <v>6</v>
@@ -8119,10 +8102,10 @@
     </row>
     <row r="6" ht="16.5" spans="2:13">
       <c r="B6" s="28" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D6" s="29">
         <f>VLOOKUP(C6,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8144,21 +8127,21 @@
         <v>3</v>
       </c>
       <c r="K6" s="29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L6" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M6" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" spans="2:16">
       <c r="B7" s="26" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D7" s="27">
         <f>VLOOKUP(C7,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8180,25 +8163,25 @@
         <v>4</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L7" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O7" s="35" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="P7" s="36"/>
     </row>
     <row r="8" ht="15" customHeight="1" spans="2:16">
       <c r="B8" s="28" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D8" s="29">
         <f>VLOOKUP(C8,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8220,13 +8203,13 @@
         <v>10</v>
       </c>
       <c r="K8" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L8" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M8" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O8" s="38" t="s">
         <v>4</v>
@@ -8238,10 +8221,10 @@
     </row>
     <row r="9" ht="15" spans="2:16">
       <c r="B9" s="26" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D9" s="27">
         <f>VLOOKUP(C9,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8263,13 +8246,13 @@
         <v>8</v>
       </c>
       <c r="K9" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L9" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M9" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O9" s="41" t="s">
         <v>9</v>
@@ -8281,10 +8264,10 @@
     </row>
     <row r="10" ht="15" spans="2:16">
       <c r="B10" s="28" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D10" s="29">
         <f>VLOOKUP(C10,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8306,13 +8289,13 @@
         <v>3</v>
       </c>
       <c r="K10" s="29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L10" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M10" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O10" s="38" t="s">
         <v>10</v>
@@ -8324,10 +8307,10 @@
     </row>
     <row r="11" ht="15" spans="2:16">
       <c r="B11" s="26" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D11" s="27">
         <f>VLOOKUP(C11,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8349,13 +8332,13 @@
         <v>3</v>
       </c>
       <c r="K11" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L11" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O11" s="41" t="s">
         <v>12</v>
@@ -8367,10 +8350,10 @@
     </row>
     <row r="12" ht="15" spans="2:16">
       <c r="B12" s="28" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D12" s="29">
         <f>VLOOKUP(C12,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8392,13 +8375,13 @@
         <v>3</v>
       </c>
       <c r="K12" s="29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L12" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M12" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="O12" s="38" t="s">
         <v>14</v>
@@ -8410,10 +8393,10 @@
     </row>
     <row r="13" ht="15.75" spans="2:16">
       <c r="B13" s="26" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D13" s="27">
         <f>VLOOKUP(C13,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8435,13 +8418,13 @@
         <v>4</v>
       </c>
       <c r="K13" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="L13" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="M13" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="L13" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="M13" s="37" t="s">
-        <v>141</v>
       </c>
       <c r="O13" s="45" t="s">
         <v>16</v>
@@ -8453,10 +8436,10 @@
     </row>
     <row r="14" ht="15.75" spans="2:13">
       <c r="B14" s="28" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D14" s="29">
         <f>VLOOKUP(C14,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8480,21 +8463,21 @@
         <v>11</v>
       </c>
       <c r="K14" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L14" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M14" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" ht="14.25" spans="2:13">
       <c r="B15" s="26" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D15" s="27">
         <f>VLOOKUP(C15,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8516,21 +8499,21 @@
         <v>4</v>
       </c>
       <c r="K15" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L15" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" ht="15" spans="2:13">
       <c r="B16" s="28" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D16" s="29">
         <f>VLOOKUP(C16,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8552,21 +8535,21 @@
         <v>3</v>
       </c>
       <c r="K16" s="29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L16" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M16" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" ht="14.25" spans="2:13">
       <c r="B17" s="26" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D17" s="27">
         <f>VLOOKUP(C17,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8588,21 +8571,21 @@
         <v>6</v>
       </c>
       <c r="K17" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L17" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" ht="15" spans="2:13">
       <c r="B18" s="28" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D18" s="29">
         <f>VLOOKUP(C18,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8624,21 +8607,21 @@
         <v>10</v>
       </c>
       <c r="K18" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L18" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M18" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" ht="14.25" spans="2:13">
       <c r="B19" s="26" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D19" s="27">
         <f>VLOOKUP(C19,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8660,21 +8643,21 @@
         <v>3</v>
       </c>
       <c r="K19" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="L19" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L19" s="27" t="s">
-        <v>141</v>
-      </c>
       <c r="M19" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" ht="15" spans="2:13">
       <c r="B20" s="28" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D20" s="29">
         <f>VLOOKUP(C20,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8696,21 +8679,21 @@
         <v>4</v>
       </c>
       <c r="K20" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="L20" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L20" s="29" t="s">
-        <v>141</v>
-      </c>
       <c r="M20" s="40" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" ht="14.25" spans="2:13">
       <c r="B21" s="26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D21" s="27">
         <f>VLOOKUP(C21,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8732,21 +8715,21 @@
         <v>7</v>
       </c>
       <c r="K21" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L21" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M21" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" ht="15" spans="2:13">
       <c r="B22" s="28" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D22" s="29">
         <f>VLOOKUP(C22,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8770,21 +8753,21 @@
         <v>12</v>
       </c>
       <c r="K22" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L22" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M22" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23" ht="14.25" spans="2:13">
       <c r="B23" s="26" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D23" s="27">
         <f>VLOOKUP(C23,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8806,21 +8789,21 @@
         <v>8</v>
       </c>
       <c r="K23" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="L23" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L23" s="27" t="s">
-        <v>141</v>
-      </c>
       <c r="M23" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" ht="15" spans="2:13">
       <c r="B24" s="28" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D24" s="29">
         <f>VLOOKUP(C24,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8842,21 +8825,21 @@
         <v>10</v>
       </c>
       <c r="K24" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L24" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M24" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" ht="14.25" spans="2:13">
       <c r="B25" s="26" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D25" s="27">
         <f>VLOOKUP(C25,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8878,21 +8861,21 @@
         <v>10</v>
       </c>
       <c r="K25" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L25" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M25" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" ht="15" spans="2:13">
       <c r="B26" s="30" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D26" s="29">
         <f>VLOOKUP(C26,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8914,21 +8897,21 @@
         <v>10</v>
       </c>
       <c r="K26" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L26" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M26" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="27" ht="14.25" spans="2:13">
       <c r="B27" s="26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D27" s="27">
         <f>VLOOKUP(C27,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8952,21 +8935,21 @@
         <v>10</v>
       </c>
       <c r="K27" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L27" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M27" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="28" ht="15" spans="2:13">
       <c r="B28" s="28" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D28" s="29">
         <f>VLOOKUP(C28,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -8988,21 +8971,21 @@
         <v>4</v>
       </c>
       <c r="K28" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="L28" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L28" s="29" t="s">
-        <v>141</v>
-      </c>
       <c r="M28" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" ht="14.25" spans="2:13">
       <c r="B29" s="26" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D29" s="27">
         <f>VLOOKUP(C29,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9024,21 +9007,21 @@
         <v>4</v>
       </c>
       <c r="K29" s="27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L29" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M29" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30" ht="15" spans="2:13">
       <c r="B30" s="28" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D30" s="29">
         <f>VLOOKUP(C30,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9060,21 +9043,21 @@
         <v>6</v>
       </c>
       <c r="K30" s="29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L30" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M30" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" ht="14.25" spans="2:13">
       <c r="B31" s="26" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D31" s="27">
         <f>VLOOKUP(C31,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9096,21 +9079,21 @@
         <v>8</v>
       </c>
       <c r="K31" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L31" s="27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M31" s="37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" ht="15" spans="2:13">
       <c r="B32" s="28" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D32" s="29">
         <f>VLOOKUP(C32,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9132,21 +9115,21 @@
         <v>6</v>
       </c>
       <c r="K32" s="29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L32" s="29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M32" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="33" ht="14.25" spans="2:13">
       <c r="B33" s="31" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C33" s="32" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D33" s="32">
         <f>VLOOKUP(C33,Clebina!$B$3:$D$8,3,FALSE)</f>
@@ -9168,13 +9151,13 @@
         <v>8</v>
       </c>
       <c r="K33" s="32" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L33" s="32" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M33" s="47" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -9207,7 +9190,7 @@
     <row r="1" ht="14.25"/>
     <row r="2" ht="15.75" spans="2:13">
       <c r="B2" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C2" s="2"/>
       <c r="E2" s="1">
@@ -9217,16 +9200,16 @@
         <v>2</v>
       </c>
       <c r="H2" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="I2" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="L2" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="M2" s="2">
         <f>12+Clebina!D5</f>
@@ -9257,7 +9240,7 @@
         <v>0</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="M3" s="4">
         <v>4</v>
@@ -9287,7 +9270,7 @@
         <v>1</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="M4" s="8">
         <v>1</v>
@@ -9403,7 +9386,7 @@
     </row>
     <row r="12" ht="15.75" spans="2:10">
       <c r="B12" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C12" s="2">
         <f>3+Clebina!D5</f>
@@ -9422,7 +9405,7 @@
     </row>
     <row r="13" ht="14.25" spans="2:10">
       <c r="B13" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C13" s="4">
         <f>SUM(M3:M4)</f>
@@ -9467,16 +9450,16 @@
     </row>
     <row r="16" ht="15.75" spans="2:10">
       <c r="B16" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H16" s="16">
         <v>91000</v>
@@ -9644,8 +9627,8 @@
   <commentList sheetStid="9">
     <comment s:ref="D5" rgbClr="217AA0"/>
     <comment s:ref="D6" rgbClr="E3E4E0"/>
-    <comment s:ref="D7" rgbClr="BDBBC0"/>
-    <comment s:ref="D9" rgbClr="77DE00"/>
+    <comment s:ref="D7" rgbClr="77DE00"/>
+    <comment s:ref="D9" rgbClr="BDBBC0"/>
   </commentList>
   <commentList sheetStid="6"/>
 </comments>

</xml_diff>